<commit_message>
feat: Refactor analysis engine and add new plotting strategies
</commit_message>
<xml_diff>
--- a/LifeTables/Tables For Testing/UK-annuity-tables-a(55).xlsx
+++ b/LifeTables/Tables For Testing/UK-annuity-tables-a(55).xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B654DDAE-3598-4D5B-8929-5D9EDA97F0CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70F6E5F-7CA3-4ABB-B391-94986D4E64F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19290" yWindow="-12840" windowWidth="19380" windowHeight="20970" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="7" r:id="rId1"/>
@@ -696,14 +696,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.00000_-;\-* #,##0.00000_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="170" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="170" formatCode="0.000%"/>
   </numFmts>
   <fonts count="28" x14ac:knownFonts="1">
     <font>
@@ -1081,7 +1082,7 @@
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1216,14 +1217,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1984,17 +1986,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
       <c r="J1" s="1" t="s">
         <v>36</v>
       </c>
@@ -2105,7 +2107,7 @@
         <f>(1+L$2)^(0)</f>
         <v>1</v>
       </c>
-      <c r="Q3" s="63">
+      <c r="Q3" s="62">
         <f>B3*P3/B$3</f>
         <v>1</v>
       </c>
@@ -2121,11 +2123,11 @@
         <f>(1+L$2)^-A3</f>
         <v>9.506040102090417E-2</v>
       </c>
-      <c r="U3" s="64">
+      <c r="U3" s="63">
         <f>T3*J3</f>
         <v>81743.959804291837</v>
       </c>
-      <c r="V3" s="65">
+      <c r="V3" s="64">
         <f t="shared" ref="V3:V45" si="0">V4+U3</f>
         <v>1032009.9562406</v>
       </c>
@@ -2133,7 +2135,7 @@
         <f>V4/U3</f>
         <v>11.624907806171827</v>
       </c>
-      <c r="X3" s="66">
+      <c r="X3" s="65">
         <f>(G3-W3)/G3</f>
         <v>7.9306518858918215E-6</v>
       </c>
@@ -2184,7 +2186,7 @@
         <f>(1+L$2)^(-(A4-A$3))</f>
         <v>0.96153846153846145</v>
       </c>
-      <c r="Q4" s="63">
+      <c r="Q4" s="62">
         <f>B4*P4/B$3</f>
         <v>0.94805771726540722</v>
       </c>
@@ -2200,11 +2202,11 @@
         <f t="shared" ref="T4:T7" si="6">(1+L$2)^-A4</f>
         <v>9.1404231750869397E-2</v>
       </c>
-      <c r="U4" s="64">
+      <c r="U4" s="63">
         <f t="shared" ref="U4:U7" si="7">T4*J4</f>
         <v>77497.989892149679</v>
       </c>
-      <c r="V4" s="65">
+      <c r="V4" s="64">
         <f t="shared" si="0"/>
         <v>950265.99643630814</v>
       </c>
@@ -2212,7 +2214,7 @@
         <f t="shared" ref="W4:W46" si="8">V5/U4</f>
         <v>11.261814761373151</v>
       </c>
-      <c r="X4" s="66">
+      <c r="X4" s="65">
         <f t="shared" ref="X4:X47" si="9">(G4-W4)/G4</f>
         <v>1.6448111068188357E-5</v>
       </c>
@@ -2263,7 +2265,7 @@
         <f t="shared" ref="P5:P47" si="12">(1+L$2)^(-(A5-A$3))</f>
         <v>0.92455621301775137</v>
       </c>
-      <c r="Q5" s="63">
+      <c r="Q5" s="62">
         <f t="shared" ref="Q5:Q47" si="13">B5*P5/B$3</f>
         <v>0.89750062555993149</v>
       </c>
@@ -2279,11 +2281,11 @@
         <f t="shared" si="6"/>
         <v>8.7888684375835968E-2</v>
       </c>
-      <c r="U5" s="64">
+      <c r="U5" s="63">
         <f t="shared" si="7"/>
         <v>73365.260546554855</v>
       </c>
-      <c r="V5" s="65">
+      <c r="V5" s="64">
         <f t="shared" si="0"/>
         <v>872768.00654415844</v>
       </c>
@@ -2291,7 +2293,7 @@
         <f t="shared" si="8"/>
         <v>10.896202644715375</v>
       </c>
-      <c r="X5" s="66">
+      <c r="X5" s="65">
         <f t="shared" si="9"/>
         <v>-1.8598083275902522E-5</v>
       </c>
@@ -2342,7 +2344,7 @@
         <f t="shared" si="12"/>
         <v>0.88899635867091487</v>
       </c>
-      <c r="Q6" s="63">
+      <c r="Q6" s="62">
         <f t="shared" si="13"/>
         <v>0.84825877323998033</v>
       </c>
@@ -2358,11 +2360,11 @@
         <f t="shared" si="6"/>
         <v>8.4508350361380741E-2</v>
       </c>
-      <c r="U6" s="64">
+      <c r="U6" s="63">
         <f t="shared" si="7"/>
         <v>69340.047309260219</v>
       </c>
-      <c r="V6" s="65">
+      <c r="V6" s="64">
         <f t="shared" si="0"/>
         <v>799402.74599760363</v>
       </c>
@@ -2370,7 +2372,7 @@
         <f t="shared" si="8"/>
         <v>10.528730899652055</v>
       </c>
-      <c r="X6" s="66">
+      <c r="X6" s="65">
         <f t="shared" si="9"/>
         <v>2.5558015760705968E-5</v>
       </c>
@@ -2421,7 +2423,7 @@
         <f t="shared" si="12"/>
         <v>0.85480419102972571</v>
       </c>
-      <c r="Q7" s="63">
+      <c r="Q7" s="62">
         <f t="shared" si="13"/>
         <v>0.80027527902095319</v>
       </c>
@@ -2437,11 +2439,11 @@
         <f t="shared" si="6"/>
         <v>8.1258029193635312E-2</v>
       </c>
-      <c r="U7" s="64">
+      <c r="U7" s="63">
         <f t="shared" si="7"/>
         <v>65417.667517718117</v>
       </c>
-      <c r="V7" s="65">
+      <c r="V7" s="64">
         <f t="shared" si="0"/>
         <v>730062.6986883434</v>
       </c>
@@ -2449,7 +2451,7 @@
         <f t="shared" si="8"/>
         <v>10.160023375804537</v>
       </c>
-      <c r="X7" s="66">
+      <c r="X7" s="65">
         <f t="shared" si="9"/>
         <v>-2.3007681630398752E-6</v>
       </c>
@@ -2500,7 +2502,7 @@
         <f t="shared" si="12"/>
         <v>0.82192710675935154</v>
       </c>
-      <c r="Q8" s="63">
+      <c r="Q8" s="62">
         <f t="shared" si="13"/>
         <v>0.75349021194175358</v>
       </c>
@@ -2516,11 +2518,11 @@
         <f t="shared" ref="T8:T24" si="14">(1+L$2)^-A8</f>
         <v>7.8132720378495488E-2</v>
       </c>
-      <c r="U8" s="64">
+      <c r="U8" s="63">
         <f t="shared" ref="U8:U24" si="15">T8*J8</f>
         <v>61593.250032066891</v>
       </c>
-      <c r="V8" s="65">
+      <c r="V8" s="64">
         <f t="shared" si="0"/>
         <v>664645.03117062524</v>
       </c>
@@ -2528,7 +2530,7 @@
         <f t="shared" si="8"/>
         <v>9.7908745004459981</v>
       </c>
-      <c r="X8" s="66">
+      <c r="X8" s="65">
         <f t="shared" si="9"/>
         <v>1.2817848432470368E-5</v>
       </c>
@@ -2579,7 +2581,7 @@
         <f t="shared" si="12"/>
         <v>0.79031452573014571</v>
       </c>
-      <c r="Q9" s="63">
+      <c r="Q9" s="62">
         <f t="shared" si="13"/>
         <v>0.70786747802525374</v>
       </c>
@@ -2592,11 +2594,11 @@
         <f t="shared" si="14"/>
         <v>7.5127615748553353E-2</v>
       </c>
-      <c r="U9" s="64">
+      <c r="U9" s="63">
         <f t="shared" si="15"/>
         <v>57863.897191182994</v>
       </c>
-      <c r="V9" s="65">
+      <c r="V9" s="64">
         <f t="shared" si="0"/>
         <v>603051.78113855841</v>
       </c>
@@ -2604,7 +2606,7 @@
         <f t="shared" si="8"/>
         <v>9.4219005357704884</v>
       </c>
-      <c r="X9" s="66">
+      <c r="X9" s="65">
         <f t="shared" si="9"/>
         <v>1.0556594089602642E-5</v>
       </c>
@@ -2655,7 +2657,7 @@
         <f t="shared" si="12"/>
         <v>0.75991781320206331</v>
       </c>
-      <c r="Q10" s="63">
+      <c r="Q10" s="62">
         <f t="shared" si="13"/>
         <v>0.663367009868709</v>
       </c>
@@ -2668,11 +2670,11 @@
         <f t="shared" si="14"/>
         <v>7.2238092065916693E-2</v>
       </c>
-      <c r="U10" s="64">
+      <c r="U10" s="63">
         <f t="shared" si="15"/>
         <v>54226.261038914206</v>
       </c>
-      <c r="V10" s="65">
+      <c r="V10" s="64">
         <f t="shared" si="0"/>
         <v>545187.88394737546</v>
       </c>
@@ -2680,7 +2682,7 @@
         <f t="shared" si="8"/>
         <v>9.0539456990430178</v>
       </c>
-      <c r="X10" s="66">
+      <c r="X10" s="65">
         <f t="shared" si="9"/>
         <v>5.9974549351054627E-6</v>
       </c>
@@ -2731,7 +2733,7 @@
         <f t="shared" si="12"/>
         <v>0.73069020500198378</v>
       </c>
-      <c r="Q11" s="63">
+      <c r="Q11" s="62">
         <f t="shared" si="13"/>
         <v>0.61997387731283338</v>
       </c>
@@ -2744,11 +2746,11 @@
         <f t="shared" si="14"/>
         <v>6.9459703909535264E-2</v>
       </c>
-      <c r="U11" s="64">
+      <c r="U11" s="63">
         <f t="shared" si="15"/>
         <v>50679.133598070606</v>
       </c>
-      <c r="V11" s="65">
+      <c r="V11" s="64">
         <f t="shared" si="0"/>
         <v>490961.62290846126</v>
       </c>
@@ -2756,7 +2758,7 @@
         <f t="shared" si="8"/>
         <v>8.6876483091090684</v>
       </c>
-      <c r="X11" s="66">
+      <c r="X11" s="65">
         <f t="shared" si="9"/>
         <v>4.0480074923139096E-5</v>
       </c>
@@ -2807,7 +2809,7 @@
         <f t="shared" si="12"/>
         <v>0.70258673557883045</v>
       </c>
-      <c r="Q12" s="63">
+      <c r="Q12" s="62">
         <f t="shared" si="13"/>
         <v>0.57767258622505047</v>
       </c>
@@ -2820,11 +2822,11 @@
         <f t="shared" si="14"/>
         <v>6.6788176836091603E-2</v>
       </c>
-      <c r="U12" s="64">
+      <c r="U12" s="63">
         <f t="shared" si="15"/>
         <v>47221.257328725333</v>
       </c>
-      <c r="V12" s="65">
+      <c r="V12" s="64">
         <f t="shared" si="0"/>
         <v>440282.48931039067</v>
       </c>
@@ -2832,7 +2834,7 @@
         <f t="shared" si="8"/>
         <v>8.3238196993657958</v>
       </c>
-      <c r="X12" s="66">
+      <c r="X12" s="65">
         <f t="shared" si="9"/>
         <v>2.1660335680447471E-5</v>
       </c>
@@ -2883,7 +2885,7 @@
         <f t="shared" si="12"/>
         <v>0.67556416882579851</v>
       </c>
-      <c r="Q13" s="63">
+      <c r="Q13" s="62">
         <f t="shared" si="13"/>
         <v>0.5364582036881469</v>
       </c>
@@ -2896,11 +2898,11 @@
         <f t="shared" si="14"/>
         <v>6.4219400803934235E-2</v>
       </c>
-      <c r="U13" s="64">
+      <c r="U13" s="63">
         <f t="shared" si="15"/>
         <v>43852.202238541278</v>
       </c>
-      <c r="V13" s="65">
+      <c r="V13" s="64">
         <f t="shared" si="0"/>
         <v>393061.23198166536</v>
       </c>
@@ -2908,7 +2910,7 @@
         <f t="shared" si="8"/>
         <v>7.9633179616281078</v>
       </c>
-      <c r="X13" s="66">
+      <c r="X13" s="65">
         <f t="shared" si="9"/>
         <v>-3.992987920478591E-5</v>
       </c>
@@ -2959,7 +2961,7 @@
         <f t="shared" si="12"/>
         <v>0.6495809315632679</v>
       </c>
-      <c r="Q14" s="63">
+      <c r="Q14" s="62">
         <f t="shared" si="13"/>
         <v>0.49634795070512722</v>
       </c>
@@ -2972,11 +2974,11 @@
         <f t="shared" si="14"/>
         <v>6.1749423849936765E-2</v>
       </c>
-      <c r="U14" s="64">
+      <c r="U14" s="63">
         <f t="shared" si="15"/>
         <v>40573.40680962881</v>
       </c>
-      <c r="V14" s="65">
+      <c r="V14" s="64">
         <f t="shared" si="0"/>
         <v>349209.02974312409</v>
       </c>
@@ -2984,7 +2986,7 @@
         <f t="shared" si="8"/>
         <v>7.6068451530732784</v>
       </c>
-      <c r="X14" s="66">
+      <c r="X14" s="65">
         <f t="shared" si="9"/>
         <v>2.0355846815019349E-5</v>
       </c>
@@ -3035,7 +3037,7 @@
         <f t="shared" si="12"/>
         <v>0.62459704958006512</v>
       </c>
-      <c r="Q15" s="63">
+      <c r="Q15" s="62">
         <f t="shared" si="13"/>
         <v>0.45735574849273802</v>
       </c>
@@ -3048,11 +3050,11 @@
         <f t="shared" si="14"/>
         <v>5.937444600955457E-2</v>
       </c>
-      <c r="U15" s="64">
+      <c r="U15" s="63">
         <f t="shared" si="15"/>
         <v>37386.053601603155</v>
       </c>
-      <c r="V15" s="65">
+      <c r="V15" s="64">
         <f t="shared" si="0"/>
         <v>308635.62293349527</v>
       </c>
@@ -3060,7 +3062,7 @@
         <f t="shared" si="8"/>
         <v>7.2553677963020053</v>
       </c>
-      <c r="X15" s="66">
+      <c r="X15" s="65">
         <f t="shared" si="9"/>
         <v>-5.0695561958022327E-5</v>
       </c>
@@ -3111,7 +3113,7 @@
         <f t="shared" si="12"/>
         <v>0.600574086134678</v>
       </c>
-      <c r="Q16" s="63">
+      <c r="Q16" s="62">
         <f t="shared" si="13"/>
         <v>0.41952731107009711</v>
       </c>
@@ -3124,11 +3126,11 @@
         <f t="shared" si="14"/>
         <v>5.7090813470725546E-2</v>
       </c>
-      <c r="U16" s="64">
+      <c r="U16" s="63">
         <f t="shared" si="15"/>
         <v>34293.795591209018</v>
       </c>
-      <c r="V16" s="65">
+      <c r="V16" s="64">
         <f t="shared" si="0"/>
         <v>271249.56933189213</v>
       </c>
@@ -3136,7 +3138,7 @@
         <f t="shared" si="8"/>
         <v>6.90958144631343</v>
       </c>
-      <c r="X16" s="66">
+      <c r="X16" s="65">
         <f t="shared" si="9"/>
         <v>6.057216882347001E-5</v>
       </c>
@@ -3187,7 +3189,7 @@
         <f t="shared" si="12"/>
         <v>0.57747508282180582</v>
       </c>
-      <c r="Q17" s="63">
+      <c r="Q17" s="62">
         <f t="shared" si="13"/>
         <v>0.38291949693379929</v>
       </c>
@@ -3200,11 +3202,11 @@
         <f t="shared" si="14"/>
         <v>5.4895012952620711E-2</v>
       </c>
-      <c r="U17" s="64">
+      <c r="U17" s="63">
         <f t="shared" si="15"/>
         <v>31301.332177841501</v>
       </c>
-      <c r="V17" s="65">
+      <c r="V17" s="64">
         <f t="shared" si="0"/>
         <v>236955.77374068313</v>
       </c>
@@ -3212,7 +3214,7 @@
         <f t="shared" si="8"/>
         <v>6.5701498068643316</v>
       </c>
-      <c r="X17" s="66">
+      <c r="X17" s="65">
         <f t="shared" si="9"/>
         <v>-2.2801653627291219E-5</v>
       </c>
@@ -3263,7 +3265,7 @@
         <f t="shared" si="12"/>
         <v>0.55526450271327477</v>
       </c>
-      <c r="Q18" s="63">
+      <c r="Q18" s="62">
         <f t="shared" si="13"/>
         <v>0.34759143576239832</v>
       </c>
@@ -3276,11 +3278,11 @@
         <f t="shared" si="14"/>
         <v>5.2783666300596846E-2</v>
       </c>
-      <c r="U18" s="64">
+      <c r="U18" s="63">
         <f t="shared" si="15"/>
         <v>28413.483310087762</v>
       </c>
-      <c r="V18" s="65">
+      <c r="V18" s="64">
         <f t="shared" si="0"/>
         <v>205654.44156284162</v>
       </c>
@@ -3288,7 +3290,7 @@
         <f t="shared" si="8"/>
         <v>6.2379172704188379</v>
       </c>
-      <c r="X18" s="66">
+      <c r="X18" s="65">
         <f t="shared" si="9"/>
         <v>1.3262196403095641E-5</v>
       </c>
@@ -3339,7 +3341,7 @@
         <f t="shared" si="12"/>
         <v>0.53390817568584104</v>
       </c>
-      <c r="Q19" s="63">
+      <c r="Q19" s="62">
         <f t="shared" si="13"/>
         <v>0.31362097891239615</v>
       </c>
@@ -3352,11 +3354,11 @@
         <f t="shared" si="14"/>
         <v>5.0753525289035421E-2</v>
       </c>
-      <c r="U19" s="64">
+      <c r="U19" s="63">
         <f t="shared" si="15"/>
         <v>25636.611729667256</v>
       </c>
-      <c r="V19" s="65">
+      <c r="V19" s="64">
         <f t="shared" si="0"/>
         <v>177240.95825275386</v>
       </c>
@@ -3364,7 +3366,7 @@
         <f t="shared" si="8"/>
         <v>5.9135874943897786</v>
       </c>
-      <c r="X19" s="66">
+      <c r="X19" s="65">
         <f t="shared" si="9"/>
         <v>6.9750694998495658E-5</v>
       </c>
@@ -3415,7 +3417,7 @@
         <f t="shared" si="12"/>
         <v>0.51337324585177024</v>
       </c>
-      <c r="Q20" s="63">
+      <c r="Q20" s="62">
         <f t="shared" si="13"/>
         <v>0.28109512928772701</v>
       </c>
@@ -3428,11 +3430,11 @@
         <f t="shared" si="14"/>
         <v>4.8801466624072518E-2</v>
       </c>
-      <c r="U20" s="64">
+      <c r="U20" s="63">
         <f t="shared" si="15"/>
         <v>22977.799286242342</v>
       </c>
-      <c r="V20" s="65">
+      <c r="V20" s="64">
         <f t="shared" si="0"/>
         <v>151604.3465230866</v>
       </c>
@@ -3440,7 +3442,7 @@
         <f t="shared" si="8"/>
         <v>5.5978619028958851</v>
       </c>
-      <c r="X20" s="66">
+      <c r="X20" s="65">
         <f t="shared" si="9"/>
         <v>2.4669007523172657E-5</v>
       </c>
@@ -3491,7 +3493,7 @@
         <f t="shared" si="12"/>
         <v>0.49362812101131748</v>
       </c>
-      <c r="Q21" s="63">
+      <c r="Q21" s="62">
         <f t="shared" si="13"/>
         <v>0.25011250731131301</v>
       </c>
@@ -3504,11 +3506,11 @@
         <f t="shared" si="14"/>
         <v>4.6924487138531264E-2</v>
       </c>
-      <c r="U21" s="64">
+      <c r="U21" s="63">
         <f t="shared" si="15"/>
         <v>20445.159736067377</v>
       </c>
-      <c r="V21" s="65">
+      <c r="V21" s="64">
         <f t="shared" si="0"/>
         <v>128626.54723684427</v>
       </c>
@@ -3516,7 +3518,7 @@
         <f t="shared" si="8"/>
         <v>5.2912957833209653</v>
       </c>
-      <c r="X21" s="66">
+      <c r="X21" s="65">
         <f t="shared" si="9"/>
         <v>-5.590310356547254E-5</v>
       </c>
@@ -3567,7 +3569,7 @@
         <f t="shared" si="12"/>
         <v>0.47464242404934376</v>
       </c>
-      <c r="Q22" s="63">
+      <c r="Q22" s="62">
         <f t="shared" si="13"/>
         <v>0.22077499594574421</v>
       </c>
@@ -3580,11 +3582,11 @@
         <f t="shared" si="14"/>
         <v>4.5119699171664682E-2</v>
       </c>
-      <c r="U22" s="64">
+      <c r="U22" s="63">
         <f t="shared" si="15"/>
         <v>18046.981816641553</v>
       </c>
-      <c r="V22" s="65">
+      <c r="V22" s="64">
         <f t="shared" si="0"/>
         <v>108181.38750077689</v>
       </c>
@@ -3592,7 +3594,7 @@
         <f t="shared" si="8"/>
         <v>4.9944310134462624</v>
       </c>
-      <c r="X22" s="66">
+      <c r="X22" s="65">
         <f t="shared" si="9"/>
         <v>-8.6306256760636376E-5</v>
       </c>
@@ -3643,7 +3645,7 @@
         <f t="shared" si="12"/>
         <v>0.45638694620129205</v>
       </c>
-      <c r="Q23" s="63">
+      <c r="Q23" s="62">
         <f t="shared" si="13"/>
         <v>0.19318252124016125</v>
       </c>
@@ -3656,11 +3658,11 @@
         <f t="shared" si="14"/>
         <v>4.3384326126600647E-2</v>
       </c>
-      <c r="U23" s="64">
+      <c r="U23" s="63">
         <f t="shared" si="15"/>
         <v>15791.456146903985</v>
       </c>
-      <c r="V23" s="65">
+      <c r="V23" s="64">
         <f t="shared" si="0"/>
         <v>90134.405684135345</v>
       </c>
@@ -3668,7 +3670,7 @@
         <f t="shared" si="8"/>
         <v>4.7077957121646925</v>
       </c>
-      <c r="X23" s="66">
+      <c r="X23" s="65">
         <f t="shared" si="9"/>
         <v>4.3391638765437888E-5</v>
       </c>
@@ -3719,7 +3721,7 @@
         <f t="shared" si="12"/>
         <v>0.43883360211662686</v>
       </c>
-      <c r="Q24" s="63">
+      <c r="Q24" s="62">
         <f t="shared" si="13"/>
         <v>0.16743545554130992</v>
       </c>
@@ -3732,11 +3734,11 @@
         <f t="shared" si="14"/>
         <v>4.171569819865447E-2</v>
       </c>
-      <c r="U24" s="64">
+      <c r="U24" s="63">
         <f t="shared" si="15"/>
         <v>13686.789092555564</v>
       </c>
-      <c r="V24" s="65">
+      <c r="V24" s="64">
         <f t="shared" si="0"/>
         <v>74342.949537231354</v>
       </c>
@@ -3744,7 +3746,7 @@
         <f t="shared" si="8"/>
         <v>4.4317304836433493</v>
       </c>
-      <c r="X24" s="66">
+      <c r="X24" s="65">
         <f t="shared" si="9"/>
         <v>6.0811452312966423E-5</v>
       </c>
@@ -3795,7 +3797,7 @@
         <f t="shared" si="12"/>
         <v>0.42195538665060278</v>
       </c>
-      <c r="Q25" s="63">
+      <c r="Q25" s="62">
         <f t="shared" si="13"/>
         <v>0.14361623991750175</v>
       </c>
@@ -3808,11 +3810,11 @@
         <f t="shared" ref="T25:T47" si="16">(1+L$2)^-A25</f>
         <v>4.0111248267936987E-2</v>
       </c>
-      <c r="U25" s="64">
+      <c r="U25" s="63">
         <f t="shared" ref="U25:U47" si="17">T25*J25</f>
         <v>11739.711740398257</v>
       </c>
-      <c r="V25" s="65">
+      <c r="V25" s="64">
         <f t="shared" si="0"/>
         <v>60656.160444675785</v>
       </c>
@@ -3820,7 +3822,7 @@
         <f t="shared" si="8"/>
         <v>4.1667504097181594</v>
       </c>
-      <c r="X25" s="66">
+      <c r="X25" s="65">
         <f t="shared" si="9"/>
         <v>5.9896875891639461E-5</v>
       </c>
@@ -3871,7 +3873,7 @@
         <f t="shared" si="12"/>
         <v>0.40572633331788732</v>
       </c>
-      <c r="Q26" s="63">
+      <c r="Q26" s="62">
         <f t="shared" si="13"/>
         <v>0.12180056301547199</v>
       </c>
@@ -3884,11 +3886,11 @@
         <f t="shared" si="16"/>
         <v>3.8568507949939407E-2</v>
       </c>
-      <c r="U26" s="64">
+      <c r="U26" s="63">
         <f t="shared" si="17"/>
         <v>9956.4043742942995</v>
       </c>
-      <c r="V26" s="65">
+      <c r="V26" s="64">
         <f t="shared" si="0"/>
         <v>48916.448704277529</v>
       </c>
@@ -3896,7 +3898,7 @@
         <f t="shared" si="8"/>
         <v>3.9130636789493272</v>
       </c>
-      <c r="X26" s="66">
+      <c r="X26" s="65">
         <f t="shared" si="9"/>
         <v>-1.6273690091323896E-5</v>
       </c>
@@ -3947,7 +3949,7 @@
         <f t="shared" si="12"/>
         <v>0.39012147434412242</v>
       </c>
-      <c r="Q27" s="63">
+      <c r="Q27" s="62">
         <f t="shared" si="13"/>
         <v>0.10203852646489034</v>
       </c>
@@ -3960,11 +3962,11 @@
         <f t="shared" si="16"/>
         <v>3.7085103798018659E-2</v>
       </c>
-      <c r="U27" s="64">
+      <c r="U27" s="63">
         <f t="shared" si="17"/>
         <v>8340.9777645650502</v>
       </c>
-      <c r="V27" s="65">
+      <c r="V27" s="64">
         <f t="shared" si="0"/>
         <v>38960.044329983226</v>
       </c>
@@ -3972,7 +3974,7 @@
         <f t="shared" si="8"/>
         <v>3.6709205358989285</v>
       </c>
-      <c r="X27" s="66">
+      <c r="X27" s="65">
         <f t="shared" si="9"/>
         <v>2.1646445402149698E-5</v>
       </c>
@@ -4023,7 +4025,7 @@
         <f t="shared" si="12"/>
         <v>0.37511680225396377</v>
       </c>
-      <c r="Q28" s="63">
+      <c r="Q28" s="62">
         <f t="shared" si="13"/>
         <v>8.4355433266345189E-2</v>
       </c>
@@ -4036,11 +4038,11 @@
         <f t="shared" si="16"/>
         <v>3.5658753651941009E-2</v>
       </c>
-      <c r="U28" s="64">
+      <c r="U28" s="63">
         <f t="shared" si="17"/>
         <v>6895.50235830778</v>
       </c>
-      <c r="V28" s="65">
+      <c r="V28" s="64">
         <f t="shared" si="0"/>
         <v>30619.066565418179</v>
       </c>
@@ -4048,7 +4050,7 @@
         <f t="shared" si="8"/>
         <v>3.4404403007023814</v>
       </c>
-      <c r="X28" s="66">
+      <c r="X28" s="65">
         <f t="shared" si="9"/>
         <v>-1.2799439022716144E-4</v>
       </c>
@@ -4099,7 +4101,7 @@
         <f t="shared" si="12"/>
         <v>0.36068923293650368</v>
       </c>
-      <c r="Q29" s="63">
+      <c r="Q29" s="62">
         <f t="shared" si="13"/>
         <v>6.8744855477622616E-2</v>
       </c>
@@ -4112,11 +4114,11 @@
         <f t="shared" si="16"/>
         <v>3.4287263126866356E-2</v>
       </c>
-      <c r="U29" s="64">
+      <c r="U29" s="63">
         <f t="shared" si="17"/>
         <v>5619.4366045770912</v>
       </c>
-      <c r="V29" s="65">
+      <c r="V29" s="64">
         <f t="shared" si="0"/>
         <v>23723.564207110398</v>
       </c>
@@ -4124,7 +4126,7 @@
         <f t="shared" si="8"/>
         <v>3.2216979879775316</v>
       </c>
-      <c r="X29" s="66">
+      <c r="X29" s="65">
         <f t="shared" si="9"/>
         <v>9.3734333478702247E-5</v>
       </c>
@@ -4175,7 +4177,7 @@
         <f t="shared" si="12"/>
         <v>0.3468165701312535</v>
       </c>
-      <c r="Q30" s="63">
+      <c r="Q30" s="62">
         <f t="shared" si="13"/>
         <v>5.5166967155900554E-2</v>
       </c>
@@ -4188,11 +4190,11 @@
         <f t="shared" si="16"/>
         <v>3.2968522237371505E-2</v>
       </c>
-      <c r="U30" s="64">
+      <c r="U30" s="63">
         <f t="shared" si="17"/>
         <v>4509.5438421288418</v>
       </c>
-      <c r="V30" s="65">
+      <c r="V30" s="64">
         <f t="shared" si="0"/>
         <v>18104.127602533306</v>
       </c>
@@ -4200,7 +4202,7 @@
         <f t="shared" si="8"/>
         <v>3.0146250344440171</v>
       </c>
-      <c r="X30" s="66">
+      <c r="X30" s="65">
         <f t="shared" si="9"/>
         <v>1.2436668523483989E-4</v>
       </c>
@@ -4251,7 +4253,7 @@
         <f t="shared" si="12"/>
         <v>0.3334774712800514</v>
       </c>
-      <c r="Q31" s="63">
+      <c r="Q31" s="62">
         <f t="shared" si="13"/>
         <v>4.3544778025006919E-2</v>
       </c>
@@ -4264,11 +4266,11 @@
         <f t="shared" si="16"/>
         <v>3.1700502151318748E-2</v>
       </c>
-      <c r="U31" s="64">
+      <c r="U31" s="63">
         <f t="shared" si="17"/>
         <v>3559.5043653880439</v>
       </c>
-      <c r="V31" s="65">
+      <c r="V31" s="64">
         <f t="shared" si="0"/>
         <v>13594.583760404465</v>
       </c>
@@ -4276,7 +4278,7 @@
         <f t="shared" si="8"/>
         <v>2.8192350296281865</v>
       </c>
-      <c r="X31" s="66">
+      <c r="X31" s="65">
         <f t="shared" si="9"/>
         <v>-8.3373404819636772E-5</v>
       </c>
@@ -4327,7 +4329,7 @@
         <f t="shared" si="12"/>
         <v>0.32065141469235708</v>
       </c>
-      <c r="Q32" s="63">
+      <c r="Q32" s="62">
         <f t="shared" si="13"/>
         <v>3.3769756660864472E-2</v>
       </c>
@@ -4340,11 +4342,11 @@
         <f t="shared" si="16"/>
         <v>3.0481252068575718E-2</v>
       </c>
-      <c r="U32" s="64">
+      <c r="U32" s="63">
         <f t="shared" si="17"/>
         <v>2760.4640873654548</v>
       </c>
-      <c r="V32" s="65">
+      <c r="V32" s="64">
         <f t="shared" si="0"/>
         <v>10035.079395016421</v>
       </c>
@@ -4352,7 +4354,7 @@
         <f>V33/U32</f>
         <v>2.635287066745994</v>
       </c>
-      <c r="X32" s="66">
+      <c r="X32" s="65">
         <f t="shared" si="9"/>
         <v>-1.0894373662019482E-4</v>
       </c>
@@ -4403,7 +4405,7 @@
         <f t="shared" si="12"/>
         <v>0.30831866797342034</v>
       </c>
-      <c r="Q33" s="63">
+      <c r="Q33" s="62">
         <f t="shared" si="13"/>
         <v>2.5701229838345507E-2</v>
       </c>
@@ -4416,11 +4418,11 @@
         <f t="shared" si="16"/>
         <v>2.9308896219784344E-2</v>
       </c>
-      <c r="U33" s="64">
+      <c r="U33" s="63">
         <f t="shared" si="17"/>
         <v>2100.8989709525295</v>
       </c>
-      <c r="V33" s="65">
+      <c r="V33" s="64">
         <f t="shared" si="0"/>
         <v>7274.6153076509663</v>
       </c>
@@ -4428,7 +4430,7 @@
         <f t="shared" si="8"/>
         <v>2.4626202441104144</v>
       </c>
-      <c r="X33" s="66">
+      <c r="X33" s="65">
         <f t="shared" si="9"/>
         <v>1.5418428322603331E-4</v>
       </c>
@@ -4479,7 +4481,7 @@
         <f t="shared" si="12"/>
         <v>0.29646025766675027</v>
       </c>
-      <c r="Q34" s="63">
+      <c r="Q34" s="62">
         <f t="shared" si="13"/>
         <v>1.9173888717495643E-2</v>
       </c>
@@ -4492,11 +4494,11 @@
         <f t="shared" si="16"/>
         <v>2.8181630980561867E-2</v>
       </c>
-      <c r="U34" s="64">
+      <c r="U34" s="63">
         <f t="shared" si="17"/>
         <v>1567.3312351855184</v>
       </c>
-      <c r="V34" s="65">
+      <c r="V34" s="64">
         <f t="shared" si="0"/>
         <v>5173.7163366984369</v>
       </c>
@@ -4504,7 +4506,7 @@
         <f t="shared" si="8"/>
         <v>2.3009718817261025</v>
       </c>
-      <c r="X34" s="66">
+      <c r="X34" s="65">
         <f t="shared" si="9"/>
         <v>1.222002342360005E-5</v>
       </c>
@@ -4555,7 +4557,7 @@
         <f t="shared" si="12"/>
         <v>0.28505794006418295</v>
       </c>
-      <c r="Q35" s="63">
+      <c r="Q35" s="62">
         <f t="shared" si="13"/>
         <v>1.400566795793046E-2</v>
       </c>
@@ -4568,11 +4570,11 @@
         <f t="shared" si="16"/>
         <v>2.7097722096694102E-2</v>
       </c>
-      <c r="U35" s="64">
+      <c r="U35" s="63">
         <f t="shared" si="17"/>
         <v>1144.8751853324372</v>
       </c>
-      <c r="V35" s="65">
+      <c r="V35" s="64">
         <f t="shared" si="0"/>
         <v>3606.3851015129185</v>
       </c>
@@ -4580,7 +4582,7 @@
         <f t="shared" si="8"/>
         <v>2.150024690652836</v>
       </c>
-      <c r="X35" s="66">
+      <c r="X35" s="65">
         <f t="shared" si="9"/>
         <v>-1.1484024574910173E-5</v>
       </c>
@@ -4631,7 +4633,7 @@
         <f t="shared" si="12"/>
         <v>0.27409417313863743</v>
       </c>
-      <c r="Q36" s="63">
+      <c r="Q36" s="62">
         <f t="shared" si="13"/>
         <v>1.0006052083189644E-2</v>
       </c>
@@ -4644,11 +4646,11 @@
         <f t="shared" si="16"/>
         <v>2.6055502016052019E-2</v>
       </c>
-      <c r="U36" s="64">
+      <c r="U36" s="63">
         <f t="shared" si="17"/>
         <v>817.9362610133212</v>
       </c>
-      <c r="V36" s="65">
+      <c r="V36" s="64">
         <f t="shared" si="0"/>
         <v>2461.5099161804815</v>
       </c>
@@ -4656,7 +4658,7 @@
         <f t="shared" si="8"/>
         <v>2.009415321838131</v>
       </c>
-      <c r="X36" s="66">
+      <c r="X36" s="65">
         <f t="shared" si="9"/>
         <v>-2.0673063122503166E-4</v>
       </c>
@@ -4707,7 +4709,7 @@
         <f t="shared" si="12"/>
         <v>0.26355208955638215</v>
       </c>
-      <c r="Q37" s="63">
+      <c r="Q37" s="62">
         <f t="shared" si="13"/>
         <v>6.9845061249010285E-3</v>
       </c>
@@ -4720,11 +4722,11 @@
         <f t="shared" si="16"/>
         <v>2.5053367323126945E-2</v>
       </c>
-      <c r="U37" s="64">
+      <c r="U37" s="63">
         <f t="shared" si="17"/>
         <v>570.94310450251976</v>
       </c>
-      <c r="V37" s="65">
+      <c r="V37" s="64">
         <f t="shared" si="0"/>
         <v>1643.5736551671603</v>
       </c>
@@ -4732,7 +4734,7 @@
         <f t="shared" si="8"/>
         <v>1.8786995450260431</v>
       </c>
-      <c r="X37" s="66">
+      <c r="X37" s="65">
         <f t="shared" si="9"/>
         <v>1.5990152951406102E-4</v>
       </c>
@@ -4783,7 +4785,7 @@
         <f t="shared" si="12"/>
         <v>0.25341547072729048</v>
       </c>
-      <c r="Q38" s="63">
+      <c r="Q38" s="62">
         <f t="shared" si="13"/>
         <v>4.7587822779251538E-3</v>
       </c>
@@ -4796,11 +4798,11 @@
         <f t="shared" si="16"/>
         <v>2.4089776272237445E-2</v>
       </c>
-      <c r="U38" s="64">
+      <c r="U38" s="63">
         <f t="shared" si="17"/>
         <v>388.99341880514459</v>
       </c>
-      <c r="V38" s="65">
+      <c r="V38" s="64">
         <f t="shared" si="0"/>
         <v>1072.6305506646404</v>
       </c>
@@ -4808,7 +4810,7 @@
         <f t="shared" si="8"/>
         <v>1.7574516657875512</v>
       </c>
-      <c r="X38" s="66">
+      <c r="X38" s="65">
         <f t="shared" si="9"/>
         <v>-2.5706646986413883E-4</v>
       </c>
@@ -4859,7 +4861,7 @@
         <f t="shared" si="12"/>
         <v>0.24366872185316396</v>
       </c>
-      <c r="Q39" s="63">
+      <c r="Q39" s="62">
         <f t="shared" si="13"/>
         <v>3.1617688221147223E-3</v>
       </c>
@@ -4872,11 +4874,11 @@
         <f t="shared" si="16"/>
         <v>2.3163246415612924E-2</v>
       </c>
-      <c r="U39" s="64">
+      <c r="U39" s="63">
         <f t="shared" si="17"/>
         <v>258.4449832613372</v>
       </c>
-      <c r="V39" s="65">
+      <c r="V39" s="64">
         <f t="shared" si="0"/>
         <v>683.63713185949587</v>
       </c>
@@ -4884,7 +4886,7 @@
         <f t="shared" si="8"/>
         <v>1.6451940495521564</v>
       </c>
-      <c r="X39" s="66">
+      <c r="X39" s="65">
         <f t="shared" si="9"/>
         <v>-1.1796325359052013E-4</v>
       </c>
@@ -4935,7 +4937,7 @@
         <f t="shared" si="12"/>
         <v>0.23429684793573452</v>
       </c>
-      <c r="Q40" s="63">
+      <c r="Q40" s="62">
         <f t="shared" si="13"/>
         <v>2.0467556385661361E-3</v>
       </c>
@@ -4948,11 +4950,11 @@
         <f t="shared" si="16"/>
         <v>2.2272352322704737E-2</v>
       </c>
-      <c r="U40" s="64">
+      <c r="U40" s="63">
         <f t="shared" si="17"/>
         <v>167.3108210388082</v>
       </c>
-      <c r="V40" s="65">
+      <c r="V40" s="64">
         <f t="shared" si="0"/>
         <v>425.19214859815861</v>
       </c>
@@ -4960,7 +4962,7 @@
         <f t="shared" si="8"/>
         <v>1.5413308353769546</v>
       </c>
-      <c r="X40" s="66">
+      <c r="X40" s="65">
         <f t="shared" si="9"/>
         <v>-2.1468875856889258E-4</v>
       </c>
@@ -5011,7 +5013,7 @@
         <f t="shared" si="12"/>
         <v>0.22528543070743706</v>
       </c>
-      <c r="Q41" s="63">
+      <c r="Q41" s="62">
         <f t="shared" si="13"/>
         <v>1.290016072271501E-3</v>
       </c>
@@ -5024,11 +5026,11 @@
         <f t="shared" si="16"/>
         <v>2.141572338721609E-2</v>
       </c>
-      <c r="U41" s="64">
+      <c r="U41" s="63">
         <f t="shared" si="17"/>
         <v>105.46212378076029</v>
       </c>
-      <c r="V41" s="65">
+      <c r="V41" s="64">
         <f t="shared" si="0"/>
         <v>257.88132755935038</v>
       </c>
@@ -5036,7 +5038,7 @@
         <f t="shared" si="8"/>
         <v>1.4452506579086764</v>
       </c>
-      <c r="X41" s="66">
+      <c r="X41" s="65">
         <f t="shared" si="9"/>
         <v>-8.6610658495595591E-4</v>
       </c>
@@ -5087,7 +5089,7 @@
         <f t="shared" si="12"/>
         <v>0.21662060644945874</v>
       </c>
-      <c r="Q42" s="63">
+      <c r="Q42" s="62">
         <f t="shared" si="13"/>
         <v>7.9124626691182609E-4</v>
       </c>
@@ -5100,11 +5102,11 @@
         <f t="shared" si="16"/>
         <v>2.0592041718477009E-2</v>
       </c>
-      <c r="U42" s="64">
+      <c r="U42" s="63">
         <f t="shared" si="17"/>
         <v>64.687830174023844</v>
       </c>
-      <c r="V42" s="65">
+      <c r="V42" s="64">
         <f t="shared" si="0"/>
         <v>152.41920377859009</v>
       </c>
@@ -5112,7 +5114,7 @@
         <f t="shared" si="8"/>
         <v>1.3562268724820485</v>
       </c>
-      <c r="X42" s="66">
+      <c r="X42" s="65">
         <f t="shared" si="9"/>
         <v>-9.0544094616129718E-4</v>
       </c>
@@ -5163,7 +5165,7 @@
         <f t="shared" si="12"/>
         <v>0.20828904466294101</v>
       </c>
-      <c r="Q43" s="63">
+      <c r="Q43" s="62">
         <f t="shared" si="13"/>
         <v>4.7208721322556161E-4</v>
       </c>
@@ -5176,11 +5178,11 @@
         <f t="shared" si="16"/>
         <v>1.9800040113920201E-2</v>
       </c>
-      <c r="U43" s="64">
+      <c r="U43" s="63">
         <f t="shared" si="17"/>
         <v>38.593754679209916</v>
       </c>
-      <c r="V43" s="65">
+      <c r="V43" s="64">
         <f t="shared" si="0"/>
         <v>87.731373604566244</v>
       </c>
@@ -5188,7 +5190,7 @@
         <f t="shared" si="8"/>
         <v>1.2732013076671778</v>
       </c>
-      <c r="X43" s="66">
+      <c r="X43" s="65">
         <f t="shared" si="9"/>
         <v>-1.7319493840895785E-3</v>
       </c>
@@ -5239,7 +5241,7 @@
         <f t="shared" si="12"/>
         <v>0.20027792756052021</v>
       </c>
-      <c r="Q44" s="63">
+      <c r="Q44" s="62">
         <f t="shared" si="13"/>
         <v>2.7389517442537618E-4</v>
       </c>
@@ -5252,11 +5254,11 @@
         <f t="shared" si="16"/>
         <v>1.9038500109538652E-2</v>
       </c>
-      <c r="U44" s="64">
+      <c r="U44" s="63">
         <f t="shared" si="17"/>
         <v>22.388830839481656</v>
       </c>
-      <c r="V44" s="65">
+      <c r="V44" s="64">
         <f t="shared" si="0"/>
         <v>49.137618925356321</v>
       </c>
@@ -5264,7 +5266,7 @@
         <f t="shared" si="8"/>
         <v>1.194738049416338</v>
       </c>
-      <c r="X44" s="66">
+      <c r="X44" s="65">
         <f t="shared" si="9"/>
         <v>-3.981554131376506E-3</v>
       </c>
@@ -5315,7 +5317,7 @@
         <f t="shared" si="12"/>
         <v>0.19257493034665407</v>
       </c>
-      <c r="Q45" s="63">
+      <c r="Q45" s="62">
         <f t="shared" si="13"/>
         <v>1.5429893967415964E-4</v>
       </c>
@@ -5328,11 +5330,11 @@
         <f t="shared" si="16"/>
         <v>1.8306250105325626E-2</v>
       </c>
-      <c r="U45" s="64">
+      <c r="U45" s="63">
         <f t="shared" si="17"/>
         <v>12.615245069169472</v>
       </c>
-      <c r="V45" s="65">
+      <c r="V45" s="64">
         <f t="shared" si="0"/>
         <v>26.748788085874665</v>
       </c>
@@ -5340,7 +5342,7 @@
         <f t="shared" si="8"/>
         <v>1.1203542173941834</v>
       </c>
-      <c r="X45" s="66">
+      <c r="X45" s="65">
         <f t="shared" si="9"/>
         <v>-6.6075627980084492E-3</v>
       </c>
@@ -5391,7 +5393,7 @@
         <f t="shared" si="12"/>
         <v>0.18516820225639813</v>
       </c>
-      <c r="Q46" s="63">
+      <c r="Q46" s="62">
         <f t="shared" si="13"/>
         <v>8.4195162181249864E-5</v>
       </c>
@@ -5404,11 +5406,11 @@
         <f t="shared" si="16"/>
         <v>1.7602163562813106E-2</v>
       </c>
-      <c r="U46" s="64">
+      <c r="U46" s="63">
         <f t="shared" si="17"/>
         <v>6.8898646147002527</v>
       </c>
-      <c r="V46" s="65">
+      <c r="V46" s="64">
         <f>V47+U46</f>
         <v>14.133543016705193</v>
       </c>
@@ -5416,7 +5418,7 @@
         <f t="shared" si="8"/>
         <v>1.0513527924118842</v>
       </c>
-      <c r="X46" s="66">
+      <c r="X46" s="65">
         <f t="shared" si="9"/>
         <v>-1.3840686993138143E-2</v>
       </c>
@@ -5467,7 +5469,7 @@
         <f t="shared" si="12"/>
         <v>0.17804634832345972</v>
       </c>
-      <c r="Q47" s="63">
+      <c r="Q47" s="62">
         <f t="shared" si="13"/>
         <v>4.4515935148949247E-5</v>
       </c>
@@ -5480,11 +5482,11 @@
         <f t="shared" si="16"/>
         <v>1.6925157271935672E-2</v>
       </c>
-      <c r="U47" s="64">
+      <c r="U47" s="63">
         <f t="shared" si="17"/>
         <v>3.64367840200494</v>
       </c>
-      <c r="V47" s="64">
+      <c r="V47" s="63">
         <f>U47+3.6</f>
         <v>7.2436784020049405</v>
       </c>
@@ -5492,7 +5494,7 @@
         <f>U47/U47</f>
         <v>1</v>
       </c>
-      <c r="X47" s="66">
+      <c r="X47" s="65">
         <f t="shared" si="9"/>
         <v>-4.0582726326743014E-2</v>
       </c>
@@ -5531,17 +5533,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
       <c r="J1" s="1" t="s">
         <v>36</v>
       </c>
@@ -5580,8 +5582,9 @@
       <c r="K2" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="L2" s="56">
-        <v>0.04</v>
+      <c r="L2" s="68">
+        <f>EXP(4%)-1</f>
+        <v>4.0810774192388211E-2</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>40</v>
@@ -5655,11 +5658,11 @@
       </c>
       <c r="L4" s="57">
         <f t="shared" ref="L4:L47" si="1">G3*(1+L$2)/(1-E3)-1</f>
-        <v>12.944989661606737</v>
+        <v>12.955861044040152</v>
       </c>
       <c r="M4" s="57">
         <f t="shared" ref="M4:M47" si="2">G4-L4</f>
-        <v>1.033839326325392E-5</v>
+        <v>-1.0861044040151313E-2</v>
       </c>
       <c r="N4" s="58">
         <f t="shared" ref="N4:N47" si="3">(G4+1)/G3-1</f>
@@ -5667,7 +5670,7 @@
       </c>
       <c r="O4" s="58">
         <f>(G3*(1+L$2)-G4)/G4</f>
-        <v>6.8038624951718848E-2</v>
+        <v>6.8871257791704096E-2</v>
       </c>
       <c r="P4" s="54"/>
       <c r="Q4" s="54"/>
@@ -5703,11 +5706,11 @@
       </c>
       <c r="L5" s="57">
         <f t="shared" si="1"/>
-        <v>12.590413987341135</v>
+        <v>12.601008945922679</v>
       </c>
       <c r="M5" s="57">
         <f t="shared" si="2"/>
-        <v>-4.1398734113506919E-4</v>
+        <v>-1.1008945922679203E-2</v>
       </c>
       <c r="N5" s="58">
         <f t="shared" si="3"/>
@@ -5715,7 +5718,7 @@
       </c>
       <c r="O5" s="58">
         <f t="shared" ref="O5:O47" si="5">(G4*(1+L$2)-G5)/G5</f>
-        <v>6.9324861000794408E-2</v>
+        <v>7.0158496578273694E-2</v>
       </c>
       <c r="P5" s="54"/>
       <c r="Q5" s="54"/>
@@ -5751,11 +5754,11 @@
       </c>
       <c r="L6" s="57">
         <f t="shared" si="1"/>
-        <v>12.230134993129093</v>
+        <v>12.240449081604323</v>
       </c>
       <c r="M6" s="57">
         <f t="shared" si="2"/>
-        <v>-1.3499312909281969E-4</v>
+        <v>-1.0449081604322785E-2</v>
       </c>
       <c r="N6" s="58">
         <f t="shared" si="3"/>
@@ -5763,7 +5766,7 @@
       </c>
       <c r="O6" s="58">
         <f t="shared" si="5"/>
-        <v>7.0613246116107919E-2</v>
+        <v>7.1447886106473152E-2</v>
       </c>
       <c r="P6" s="54"/>
       <c r="Q6" s="54"/>
@@ -5799,11 +5802,11 @@
       </c>
       <c r="L7" s="57">
         <f t="shared" si="1"/>
-        <v>11.865480513437788</v>
+        <v>11.875510320719489</v>
       </c>
       <c r="M7" s="57">
         <f t="shared" si="2"/>
-        <v>5.1948656221156853E-4</v>
+        <v>-9.5103207194888739E-3</v>
       </c>
       <c r="N7" s="58">
         <f t="shared" si="3"/>
@@ -5811,7 +5814,7 @@
       </c>
       <c r="O7" s="58">
         <f t="shared" si="5"/>
-        <v>7.1902915894151445E-2</v>
+        <v>7.2738561298913609E-2</v>
       </c>
       <c r="P7" s="54"/>
       <c r="Q7" s="54"/>
@@ -5847,11 +5850,11 @@
       </c>
       <c r="L8" s="57">
         <f t="shared" si="1"/>
-        <v>11.497356854961215</v>
+        <v>11.507099676510318</v>
       </c>
       <c r="M8" s="57">
         <f t="shared" si="2"/>
-        <v>-3.5685496121473648E-4</v>
+        <v>-1.009967651031829E-2</v>
       </c>
       <c r="N8" s="58">
         <f t="shared" si="3"/>
@@ -5859,7 +5862,7 @@
       </c>
       <c r="O8" s="58">
         <f t="shared" si="5"/>
-        <v>7.337914238497005E-2</v>
+        <v>7.4215938641983031E-2</v>
       </c>
       <c r="P8" s="54"/>
       <c r="Q8" s="54"/>
@@ -5895,11 +5898,11 @@
       </c>
       <c r="L9" s="57">
         <f t="shared" si="1"/>
-        <v>11.1248085990975</v>
+        <v>11.13426098553961</v>
       </c>
       <c r="M9" s="57">
         <f t="shared" si="2"/>
-        <v>1.9140090249969433E-4</v>
+        <v>-9.2609855396101892E-3</v>
       </c>
       <c r="N9" s="58">
         <f t="shared" si="3"/>
@@ -5907,7 +5910,7 @@
       </c>
       <c r="O9" s="58">
         <f t="shared" si="5"/>
-        <v>7.4775730337078641E-2</v>
+        <v>7.5613615360888717E-2</v>
       </c>
       <c r="P9" s="54"/>
       <c r="Q9" s="54"/>
@@ -5943,11 +5946,11 @@
       </c>
       <c r="L10" s="57">
         <f t="shared" si="1"/>
-        <v>10.749890828585647</v>
+        <v>10.759050932669489</v>
       </c>
       <c r="M10" s="57">
         <f t="shared" si="2"/>
-        <v>1.0917141435307087E-4</v>
+        <v>-9.0509326694885317E-3</v>
       </c>
       <c r="N10" s="58">
         <f t="shared" si="3"/>
@@ -5955,7 +5958,7 @@
       </c>
       <c r="O10" s="58">
         <f t="shared" si="5"/>
-        <v>7.6279069767441893E-2</v>
+        <v>7.7118126780494706E-2</v>
       </c>
       <c r="P10" s="54"/>
       <c r="Q10" s="54"/>
@@ -5991,11 +5994,11 @@
       </c>
       <c r="L11" s="57">
         <f t="shared" si="1"/>
-        <v>10.372768424800366</v>
+        <v>10.381634527814631</v>
       </c>
       <c r="M11" s="57">
         <f t="shared" si="2"/>
-        <v>-7.6842480036631855E-4</v>
+        <v>-9.6345278146312552E-3</v>
       </c>
       <c r="N11" s="58">
         <f t="shared" si="3"/>
@@ -6003,7 +6006,7 @@
       </c>
       <c r="O11" s="58">
         <f t="shared" si="5"/>
-        <v>7.7902043964519843E-2</v>
+        <v>7.8742366232951583E-2</v>
       </c>
       <c r="P11" s="54"/>
       <c r="Q11" s="54"/>
@@ -6039,11 +6042,11 @@
       </c>
       <c r="L12" s="57">
         <f t="shared" si="1"/>
-        <v>9.9932227918021255</v>
+        <v>10.00179300462017</v>
       </c>
       <c r="M12" s="57">
         <f t="shared" si="2"/>
-        <v>7.7720819787430173E-4</v>
+        <v>-7.7930046201704073E-3</v>
       </c>
       <c r="N12" s="58">
         <f t="shared" si="3"/>
@@ -6051,7 +6054,7 @@
       </c>
       <c r="O12" s="58">
         <f t="shared" si="5"/>
-        <v>7.9335601360816521E-2</v>
+        <v>8.0177041217075321E-2</v>
       </c>
       <c r="P12" s="54"/>
       <c r="Q12" s="54"/>
@@ -6087,11 +6090,11 @@
       </c>
       <c r="L13" s="57">
         <f t="shared" si="1"/>
-        <v>9.6145424836601308</v>
+        <v>9.6228174808810536</v>
       </c>
       <c r="M13" s="57">
         <f t="shared" si="2"/>
-        <v>-5.4248366012998872E-4</v>
+        <v>-8.8174808810528305E-3</v>
       </c>
       <c r="N13" s="58">
         <f t="shared" si="3"/>
@@ -6099,7 +6102,7 @@
       </c>
       <c r="O13" s="58">
         <f t="shared" si="5"/>
-        <v>8.1106719367588884E-2</v>
+        <v>8.1949539970743349E-2</v>
       </c>
       <c r="P13" s="54"/>
       <c r="Q13" s="54"/>
@@ -6135,11 +6138,11 @@
       </c>
       <c r="L14" s="57">
         <f t="shared" si="1"/>
-        <v>9.2346739275076022</v>
+        <v>9.2426527827844591</v>
       </c>
       <c r="M14" s="57">
         <f t="shared" si="2"/>
-        <v>3.2607249239724467E-4</v>
+        <v>-7.6527827844596885E-3</v>
       </c>
       <c r="N14" s="58">
         <f t="shared" si="3"/>
@@ -6147,7 +6150,7 @@
       </c>
       <c r="O14" s="58">
         <f t="shared" si="5"/>
-        <v>8.2681104493773888E-2</v>
+        <v>8.3525152472725697E-2</v>
       </c>
       <c r="P14" s="54"/>
       <c r="Q14" s="54"/>
@@ -6183,11 +6186,11 @@
       </c>
       <c r="L15" s="57">
         <f t="shared" si="1"/>
-        <v>8.8566311922086189</v>
+        <v>8.8643153289341274</v>
       </c>
       <c r="M15" s="57">
         <f t="shared" si="2"/>
-        <v>3.6880779138037667E-4</v>
+        <v>-7.315328934128118E-3</v>
       </c>
       <c r="N15" s="58">
         <f t="shared" si="3"/>
@@ -6195,7 +6198,7 @@
       </c>
       <c r="O15" s="58">
         <f t="shared" si="5"/>
-        <v>8.4385232019871373E-2</v>
+        <v>8.5230608520571821E-2</v>
       </c>
       <c r="P15" s="54"/>
       <c r="Q15" s="54"/>
@@ -6231,11 +6234,11 @@
       </c>
       <c r="L16" s="57">
         <f t="shared" si="1"/>
-        <v>8.4804293903932653</v>
+        <v>8.4878202437418135</v>
       </c>
       <c r="M16" s="57">
         <f t="shared" si="2"/>
-        <v>-4.2939039326483908E-4</v>
+        <v>-7.8202437418131154E-3</v>
       </c>
       <c r="N16" s="58">
         <f t="shared" si="3"/>
@@ -6243,7 +6246,7 @@
       </c>
       <c r="O16" s="58">
         <f t="shared" si="5"/>
-        <v>8.6235849056603767E-2</v>
+        <v>8.7082668280894102E-2</v>
       </c>
       <c r="P16" s="54"/>
       <c r="Q16" s="54"/>
@@ -6279,11 +6282,11 @@
       </c>
       <c r="L17" s="57">
         <f t="shared" si="1"/>
-        <v>8.1061342915259846</v>
+        <v>8.1132333479452061</v>
       </c>
       <c r="M17" s="57">
         <f t="shared" si="2"/>
-        <v>-1.3429152598476435E-4</v>
+        <v>-7.2333479452062477E-3</v>
       </c>
       <c r="N17" s="58">
         <f t="shared" si="3"/>
@@ -6291,7 +6294,7 @@
       </c>
       <c r="O17" s="58">
         <f t="shared" si="5"/>
-        <v>8.7984209227732604E-2</v>
+        <v>8.8832391457124571E-2</v>
       </c>
       <c r="P17" s="54"/>
       <c r="Q17" s="54"/>
@@ -6327,11 +6330,11 @@
       </c>
       <c r="L18" s="57">
         <f t="shared" si="1"/>
-        <v>7.7358189467575791</v>
+        <v>7.7426293088262401</v>
       </c>
       <c r="M18" s="57">
         <f t="shared" si="2"/>
-        <v>1.8105324242068122E-4</v>
+        <v>-6.6293088262403543E-3</v>
       </c>
       <c r="N18" s="58">
         <f t="shared" si="3"/>
@@ -6339,7 +6342,7 @@
       </c>
       <c r="O18" s="58">
         <f t="shared" si="5"/>
-        <v>8.9741468459151985E-2</v>
+        <v>9.0591020631269156E-2</v>
       </c>
       <c r="P18" s="54"/>
       <c r="Q18" s="54"/>
@@ -6375,11 +6378,11 @@
       </c>
       <c r="L19" s="57">
         <f t="shared" si="1"/>
-        <v>7.3702909934560275</v>
+        <v>7.3768163933793698</v>
       </c>
       <c r="M19" s="57">
         <f t="shared" si="2"/>
-        <v>-2.9099345602734417E-4</v>
+        <v>-6.8163933793696785E-3</v>
       </c>
       <c r="N19" s="58">
         <f t="shared" si="3"/>
@@ -6387,7 +6390,7 @@
       </c>
       <c r="O19" s="58">
         <f t="shared" si="5"/>
-        <v>9.1647218453188489E-2</v>
+        <v>9.2498256330029241E-2</v>
       </c>
       <c r="P19" s="54"/>
       <c r="Q19" s="54"/>
@@ -6423,11 +6426,11 @@
       </c>
       <c r="L20" s="57">
         <f t="shared" si="1"/>
-        <v>7.0096975776955723</v>
+        <v>7.0159418623925234</v>
       </c>
       <c r="M20" s="57">
         <f t="shared" si="2"/>
-        <v>3.024223044274521E-4</v>
+        <v>-5.9418623925235892E-3</v>
       </c>
       <c r="N20" s="58">
         <f t="shared" si="3"/>
@@ -6435,7 +6438,7 @@
       </c>
       <c r="O20" s="58">
         <f t="shared" si="5"/>
-        <v>9.340941512125546E-2</v>
+        <v>9.4261826790000169E-2</v>
       </c>
       <c r="P20" s="54"/>
       <c r="Q20" s="54"/>
@@ -6471,11 +6474,11 @@
       </c>
       <c r="L21" s="57">
         <f t="shared" si="1"/>
-        <v>6.6560530958581872</v>
+        <v>6.6620216826521066</v>
       </c>
       <c r="M21" s="57">
         <f t="shared" si="2"/>
-        <v>-5.3095858187468536E-5</v>
+        <v>-6.0216826521068967E-3</v>
       </c>
       <c r="N21" s="58">
         <f t="shared" si="3"/>
@@ -6483,7 +6486,7 @@
       </c>
       <c r="O21" s="58">
         <f t="shared" si="5"/>
-        <v>9.531250000000005E-2</v>
+        <v>9.6166395295769508E-2</v>
       </c>
       <c r="P21" s="54"/>
       <c r="Q21" s="54"/>
@@ -6519,11 +6522,11 @@
       </c>
       <c r="L22" s="57">
         <f t="shared" si="1"/>
-        <v>6.3092656142759092</v>
+        <v>6.3149638488195299</v>
       </c>
       <c r="M22" s="57">
         <f t="shared" si="2"/>
-        <v>-2.6561427590898745E-4</v>
+        <v>-5.9638488195297157E-3</v>
       </c>
       <c r="N22" s="58">
         <f t="shared" si="3"/>
@@ -6531,7 +6534,7 @@
       </c>
       <c r="O22" s="58">
         <f t="shared" si="5"/>
-        <v>9.7200824219369042E-2</v>
+        <v>9.8056191634892251E-2</v>
       </c>
       <c r="P22" s="54"/>
       <c r="Q22" s="54"/>
@@ -6567,11 +6570,11 @@
       </c>
       <c r="L23" s="57">
         <f t="shared" si="1"/>
-        <v>5.970233921856078</v>
+        <v>5.9756678504894918</v>
       </c>
       <c r="M23" s="57">
         <f t="shared" si="2"/>
-        <v>7.6607814392204432E-4</v>
+        <v>-4.6678504894916983E-3</v>
       </c>
       <c r="N23" s="58">
         <f t="shared" si="3"/>
@@ -6579,7 +6582,7 @@
       </c>
       <c r="O23" s="58">
         <f t="shared" si="5"/>
-        <v>9.8871210852453595E-2</v>
+        <v>9.9727880485643558E-2</v>
       </c>
       <c r="P23" s="54"/>
       <c r="Q23" s="54"/>
@@ -6615,11 +6618,11 @@
       </c>
       <c r="L24" s="57">
         <f t="shared" si="1"/>
-        <v>5.641184963370943</v>
+        <v>5.646362368539382</v>
       </c>
       <c r="M24" s="57">
         <f t="shared" si="2"/>
-        <v>-1.8496337094298099E-4</v>
+        <v>-5.3623685393819898E-3</v>
       </c>
       <c r="N24" s="58">
         <f t="shared" si="3"/>
@@ -6627,7 +6630,7 @@
       </c>
       <c r="O24" s="58">
         <f t="shared" si="5"/>
-        <v>0.1008402765467117</v>
+        <v>0.10169848124494767</v>
       </c>
       <c r="P24" s="54"/>
       <c r="Q24" s="54"/>
@@ -6663,11 +6666,11 @@
       </c>
       <c r="L25" s="57">
         <f t="shared" si="1"/>
-        <v>5.320720565419756</v>
+        <v>5.3256481395656587</v>
       </c>
       <c r="M25" s="57">
         <f t="shared" si="2"/>
-        <v>-7.2056541975573651E-4</v>
+        <v>-5.648139565658461E-3</v>
       </c>
       <c r="N25" s="58">
         <f t="shared" si="3"/>
@@ -6675,7 +6678,7 @@
       </c>
       <c r="O25" s="58">
         <f t="shared" si="5"/>
-        <v>0.10275187969924812</v>
+        <v>0.10361157466527471</v>
       </c>
       <c r="P25" s="54"/>
       <c r="Q25" s="54"/>
@@ -6711,11 +6714,11 @@
       </c>
       <c r="L26" s="57">
         <f t="shared" si="1"/>
-        <v>5.0098629184679897</v>
+        <v>5.0145481509238401</v>
       </c>
       <c r="M26" s="57">
         <f t="shared" si="2"/>
-        <v>1.3708153201008599E-4</v>
+        <v>-4.5481509238403106E-3</v>
       </c>
       <c r="N26" s="58">
         <f t="shared" si="3"/>
@@ -6723,7 +6726,7 @@
       </c>
       <c r="O26" s="58">
         <f t="shared" si="5"/>
-        <v>0.10435129740518984</v>
+        <v>0.10521223926217689</v>
       </c>
       <c r="P26" s="54"/>
       <c r="Q26" s="54"/>
@@ -6759,11 +6762,11 @@
       </c>
       <c r="L27" s="57">
         <f t="shared" si="1"/>
-        <v>4.7106532222709339</v>
+        <v>4.7151051936692951</v>
       </c>
       <c r="M27" s="57">
         <f t="shared" si="2"/>
-        <v>3.4677772906643867E-4</v>
+        <v>-4.1051936692948487E-3</v>
       </c>
       <c r="N27" s="58">
         <f t="shared" si="3"/>
@@ -6771,7 +6774,7 @@
       </c>
       <c r="O27" s="58">
         <f t="shared" si="5"/>
-        <v>0.10600721715134782</v>
+        <v>0.10686944994775298</v>
       </c>
       <c r="P27" s="54"/>
       <c r="Q27" s="54"/>
@@ -6807,11 +6810,11 @@
       </c>
       <c r="L28" s="57">
         <f t="shared" si="1"/>
-        <v>4.4230939520056678</v>
+        <v>4.4273217449087277</v>
       </c>
       <c r="M28" s="57">
         <f t="shared" si="2"/>
-        <v>-9.3952005667752303E-5</v>
+        <v>-4.3217449087276094E-3</v>
       </c>
       <c r="N28" s="58">
         <f t="shared" si="3"/>
@@ -6819,7 +6822,7 @@
       </c>
       <c r="O28" s="58">
         <f t="shared" si="5"/>
-        <v>0.10771874293465977</v>
+        <v>0.10858231002042532</v>
       </c>
       <c r="P28" s="54"/>
       <c r="Q28" s="54"/>
@@ -6855,11 +6858,11 @@
       </c>
       <c r="L29" s="57">
         <f t="shared" si="1"/>
-        <v>4.1469364006624003</v>
+        <v>4.1509489037427088</v>
       </c>
       <c r="M29" s="57">
         <f t="shared" si="2"/>
-        <v>6.359933759991776E-5</v>
+        <v>-3.9489037427085094E-3</v>
       </c>
       <c r="N29" s="58">
         <f t="shared" si="3"/>
@@ -6867,7 +6870,7 @@
       </c>
       <c r="O29" s="58">
         <f t="shared" si="5"/>
-        <v>0.10921630094043881</v>
+        <v>0.11008103550830307</v>
       </c>
       <c r="P29" s="54"/>
       <c r="Q29" s="54"/>
@@ -6903,11 +6906,11 @@
       </c>
       <c r="L30" s="57">
         <f t="shared" si="1"/>
-        <v>3.8831321754489263</v>
+        <v>3.8869390192430364</v>
       </c>
       <c r="M30" s="57">
         <f t="shared" si="2"/>
-        <v>-1.3217544892629718E-4</v>
+        <v>-3.9390192430364124E-3</v>
       </c>
       <c r="N30" s="58">
         <f t="shared" si="3"/>
@@ -6915,7 +6918,7 @@
       </c>
       <c r="O30" s="58">
         <f t="shared" si="5"/>
-        <v>0.1107082152974506</v>
+        <v>0.1115741129476782</v>
       </c>
       <c r="P30" s="54"/>
       <c r="Q30" s="54"/>
@@ -6951,11 +6954,11 @@
       </c>
       <c r="L31" s="57">
         <f t="shared" si="1"/>
-        <v>3.6315258280576206</v>
+        <v>3.635136521916051</v>
       </c>
       <c r="M31" s="57">
         <f t="shared" si="2"/>
-        <v>4.7417194237953098E-4</v>
+        <v>-3.1365219160508495E-3</v>
       </c>
       <c r="N31" s="58">
         <f t="shared" si="3"/>
@@ -6963,7 +6966,7 @@
       </c>
       <c r="O31" s="58">
         <f t="shared" si="5"/>
-        <v>0.11187224669603536</v>
+        <v>0.11273905181416392</v>
       </c>
       <c r="P31" s="54"/>
       <c r="Q31" s="54"/>
@@ -6999,11 +7002,11 @@
       </c>
       <c r="L32" s="57">
         <f t="shared" si="1"/>
-        <v>3.393258819013945</v>
+        <v>3.3966837621590784</v>
       </c>
       <c r="M32" s="57">
         <f t="shared" si="2"/>
-        <v>-2.5881901394519957E-4</v>
+        <v>-3.6837621590786185E-3</v>
       </c>
       <c r="N32" s="58">
         <f t="shared" si="3"/>
@@ -7011,7 +7014,7 @@
       </c>
       <c r="O32" s="58">
         <f t="shared" si="5"/>
-        <v>0.11325670498084303</v>
+        <v>0.1141245894095945</v>
       </c>
       <c r="P32" s="54"/>
       <c r="Q32" s="54"/>
@@ -7047,11 +7050,11 @@
       </c>
       <c r="L33" s="57">
         <f t="shared" si="1"/>
-        <v>3.166926456001133</v>
+        <v>3.1701749525704654</v>
       </c>
       <c r="M33" s="57">
         <f t="shared" si="2"/>
-        <v>7.3543998866831828E-5</v>
+        <v>-3.1749525704656278E-3</v>
       </c>
       <c r="N33" s="58">
         <f t="shared" si="3"/>
@@ -7059,7 +7062,7 @@
       </c>
       <c r="O33" s="58">
         <f t="shared" si="5"/>
-        <v>0.11421534575307864</v>
+        <v>0.11508397752913579</v>
       </c>
       <c r="P33" s="54"/>
       <c r="Q33" s="54"/>
@@ -7095,11 +7098,11 @@
       </c>
       <c r="L34" s="57">
         <f t="shared" si="1"/>
-        <v>2.9537128178042393</v>
+        <v>2.9567950950319224</v>
       </c>
       <c r="M34" s="57">
         <f t="shared" si="2"/>
-        <v>-7.1281780423948504E-4</v>
+        <v>-3.7950950319225463E-3</v>
       </c>
       <c r="N34" s="58">
         <f t="shared" si="3"/>
@@ -7107,7 +7110,7 @@
       </c>
       <c r="O34" s="58">
         <f t="shared" si="5"/>
-        <v>0.11536742295970195</v>
+        <v>0.11623695288428493</v>
       </c>
       <c r="P34" s="54"/>
       <c r="Q34" s="54"/>
@@ -7143,11 +7146,11 @@
       </c>
       <c r="L35" s="57">
         <f t="shared" si="1"/>
-        <v>2.7521777908099065</v>
+        <v>2.7551029532310993</v>
       </c>
       <c r="M35" s="57">
         <f t="shared" si="2"/>
-        <v>8.2220919009357019E-4</v>
+        <v>-2.1029532310992138E-3</v>
       </c>
       <c r="N35" s="58">
         <f t="shared" si="3"/>
@@ -7155,7 +7158,7 @@
       </c>
       <c r="O35" s="58">
         <f t="shared" si="5"/>
-        <v>0.11555394115510351</v>
+        <v>0.11642361648751252</v>
       </c>
       <c r="P35" s="54"/>
       <c r="Q35" s="54"/>
@@ -7191,11 +7194,11 @@
       </c>
       <c r="L36" s="57">
         <f t="shared" si="1"/>
-        <v>2.5648189650879032</v>
+        <v>2.567598064335431</v>
       </c>
       <c r="M36" s="57">
         <f t="shared" si="2"/>
-        <v>-8.1896508790313405E-4</v>
+        <v>-3.5980643354309727E-3</v>
       </c>
       <c r="N36" s="58">
         <f t="shared" si="3"/>
@@ -7203,7 +7206,7 @@
       </c>
       <c r="O36" s="58">
         <f t="shared" si="5"/>
-        <v>0.11666146645865845</v>
+        <v>0.11753200520734973</v>
       </c>
       <c r="P36" s="54"/>
       <c r="Q36" s="54"/>
@@ -7239,11 +7242,11 @@
       </c>
       <c r="L37" s="57">
         <f t="shared" si="1"/>
-        <v>2.3877856970436153</v>
+        <v>2.3904267828248704</v>
       </c>
       <c r="M37" s="57">
         <f t="shared" si="2"/>
-        <v>2.1430295638458219E-4</v>
+        <v>-2.4267828248705214E-3</v>
       </c>
       <c r="N37" s="58">
         <f t="shared" si="3"/>
@@ -7251,7 +7254,7 @@
       </c>
       <c r="O37" s="58">
         <f t="shared" si="5"/>
-        <v>0.11664991624790626</v>
+        <v>0.11752044599216237</v>
       </c>
       <c r="P37" s="54"/>
       <c r="Q37" s="54"/>
@@ -7287,11 +7290,11 @@
       </c>
       <c r="L38" s="57">
         <f t="shared" si="1"/>
-        <v>2.2236760124610591</v>
+        <v>2.2261891598798327</v>
       </c>
       <c r="M38" s="57">
         <f t="shared" si="2"/>
-        <v>3.2398753894113952E-4</v>
+        <v>-2.1891598798324807E-3</v>
       </c>
       <c r="N38" s="58">
         <f t="shared" si="3"/>
@@ -7299,7 +7302,7 @@
       </c>
       <c r="O38" s="58">
         <f t="shared" si="5"/>
-        <v>0.11669064748201427</v>
+        <v>0.11756120897995627</v>
       </c>
       <c r="P38" s="54"/>
       <c r="Q38" s="54"/>
@@ -7335,11 +7338,11 @@
       </c>
       <c r="L39" s="57">
         <f t="shared" si="1"/>
-        <v>2.071170596983217</v>
+        <v>2.0735648526182704</v>
       </c>
       <c r="M39" s="57">
         <f t="shared" si="2"/>
-        <v>-1.7059698321686412E-4</v>
+        <v>-2.5648526182702192E-3</v>
       </c>
       <c r="N39" s="58">
         <f t="shared" si="3"/>
@@ -7347,7 +7350,7 @@
       </c>
       <c r="O39" s="58">
         <f t="shared" si="5"/>
-        <v>0.11683244809270892</v>
+        <v>0.11770312013706981</v>
       </c>
       <c r="P39" s="54"/>
       <c r="Q39" s="54"/>
@@ -7383,11 +7386,11 @@
       </c>
       <c r="L40" s="57">
         <f t="shared" si="1"/>
-        <v>1.9289997960155034</v>
+        <v>1.9312832166348493</v>
       </c>
       <c r="M40" s="57">
         <f t="shared" si="2"/>
-        <v>2.0398449662728524E-7</v>
+        <v>-2.2832166348492056E-3</v>
       </c>
       <c r="N40" s="58">
         <f t="shared" si="3"/>
@@ -7395,7 +7398,7 @@
       </c>
       <c r="O40" s="58">
         <f t="shared" si="5"/>
-        <v>0.11655780196993268</v>
+        <v>0.11742825990276633</v>
       </c>
       <c r="P40" s="54"/>
       <c r="Q40" s="54"/>
@@ -7431,11 +7434,11 @@
       </c>
       <c r="L41" s="57">
         <f t="shared" si="1"/>
-        <v>1.7972113775794756</v>
+        <v>1.7993920571906257</v>
       </c>
       <c r="M41" s="57">
         <f t="shared" si="2"/>
-        <v>-2.1137757947564673E-4</v>
+        <v>-2.3920571906257404E-3</v>
       </c>
       <c r="N41" s="58">
         <f t="shared" si="3"/>
@@ -7443,7 +7446,7 @@
       </c>
       <c r="O41" s="58">
         <f t="shared" si="5"/>
-        <v>0.11639398998330552</v>
+        <v>0.11726432020985925</v>
       </c>
       <c r="P41" s="54"/>
       <c r="Q41" s="54"/>
@@ -7479,11 +7482,11 @@
       </c>
       <c r="L42" s="57">
         <f t="shared" si="1"/>
-        <v>1.6745663747209343</v>
+        <v>1.6766514414444464</v>
       </c>
       <c r="M42" s="57">
         <f t="shared" si="2"/>
-        <v>-5.6637472093434837E-4</v>
+        <v>-2.6514414444465118E-3</v>
       </c>
       <c r="N42" s="58">
         <f t="shared" si="3"/>
@@ -7491,7 +7494,7 @@
       </c>
       <c r="O42" s="58">
         <f t="shared" si="5"/>
-        <v>0.1164157706093191</v>
+        <v>0.11728611781584324</v>
       </c>
       <c r="P42" s="54"/>
       <c r="Q42" s="54"/>
@@ -7527,11 +7530,11 @@
       </c>
       <c r="L43" s="57">
         <f t="shared" si="1"/>
-        <v>1.55959539526883</v>
+        <v>1.5615908317009835</v>
       </c>
       <c r="M43" s="57">
         <f t="shared" si="2"/>
-        <v>4.0460473117009954E-4</v>
+        <v>-1.5908317009833972E-3</v>
       </c>
       <c r="N43" s="58">
         <f t="shared" si="3"/>
@@ -7539,7 +7542,7 @@
       </c>
       <c r="O43" s="58">
         <f t="shared" si="5"/>
-        <v>0.11600000000000001</v>
+        <v>0.11687002307567809</v>
       </c>
       <c r="P43" s="54"/>
       <c r="Q43" s="54"/>
@@ -7575,11 +7578,11 @@
       </c>
       <c r="L44" s="57">
         <f t="shared" si="1"/>
-        <v>1.4524594128850863</v>
+        <v>1.4543713271157084</v>
       </c>
       <c r="M44" s="57">
         <f t="shared" si="2"/>
-        <v>5.4058711491378197E-4</v>
+        <v>-1.3713271157083096E-3</v>
       </c>
       <c r="N44" s="58">
         <f t="shared" si="3"/>
@@ -7587,7 +7590,7 @@
       </c>
       <c r="O44" s="58">
         <f t="shared" si="5"/>
-        <v>0.11658637302133516</v>
+        <v>0.11745685322789098</v>
       </c>
       <c r="P44" s="54"/>
       <c r="Q44" s="54"/>
@@ -7623,11 +7626,11 @@
       </c>
       <c r="L45" s="57">
         <f t="shared" si="1"/>
-        <v>1.3501088646967339</v>
+        <v>1.3519409874051944</v>
       </c>
       <c r="M45" s="57">
         <f t="shared" si="2"/>
-        <v>-1.0886469673376808E-4</v>
+        <v>-1.9409874051943277E-3</v>
       </c>
       <c r="N45" s="58">
         <f t="shared" si="3"/>
@@ -7635,7 +7638,7 @@
       </c>
       <c r="O45" s="58">
         <f t="shared" si="5"/>
-        <v>0.11934814814814809</v>
+        <v>0.12022078140854817</v>
       </c>
       <c r="P45" s="54"/>
       <c r="Q45" s="54"/>
@@ -7671,11 +7674,11 @@
       </c>
       <c r="L46" s="57">
         <f t="shared" si="1"/>
-        <v>1.2500000000000004</v>
+        <v>1.2517540787816093</v>
       </c>
       <c r="M46" s="57">
         <f t="shared" si="2"/>
-        <v>-1.000000000000334E-3</v>
+        <v>-2.7540787816091594E-3</v>
       </c>
       <c r="N46" s="58">
         <f t="shared" si="3"/>
@@ -7683,7 +7686,7 @@
       </c>
       <c r="O46" s="58">
         <f t="shared" si="5"/>
-        <v>0.12409927942353884</v>
+        <v>0.12497561662107604</v>
       </c>
       <c r="P46" s="54"/>
       <c r="Q46" s="54"/>
@@ -7719,11 +7722,11 @@
       </c>
       <c r="L47" s="57">
         <f t="shared" si="1"/>
-        <v>1.1505960264900663</v>
+        <v>1.1522726108713464</v>
       </c>
       <c r="M47" s="57">
         <f t="shared" si="2"/>
-        <v>4.0397350993370829E-4</v>
+        <v>-1.2726108713463358E-3</v>
       </c>
       <c r="N47" s="58">
         <f t="shared" si="3"/>
@@ -7731,7 +7734,7 @@
       </c>
       <c r="O47" s="58">
         <f t="shared" si="5"/>
-        <v>0.12854908774978288</v>
+        <v>0.12942889397592791</v>
       </c>
       <c r="P47" s="54"/>
       <c r="Q47" s="54"/>
@@ -8527,17 +8530,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
       <c r="J1" s="1" t="s">
         <v>36</v>
       </c>
@@ -8648,7 +8651,7 @@
         <f>(1+L$2)^(0)</f>
         <v>1</v>
       </c>
-      <c r="Q3" s="63">
+      <c r="Q3" s="62">
         <f>B3*P3/B$3</f>
         <v>1</v>
       </c>
@@ -8664,11 +8667,11 @@
         <f>(1+L$2)^-A3</f>
         <v>9.506040102090417E-2</v>
       </c>
-      <c r="U3" s="64">
+      <c r="U3" s="63">
         <f>T3*J3</f>
         <v>81743.959804291837</v>
       </c>
-      <c r="V3" s="65">
+      <c r="V3" s="64">
         <f t="shared" ref="V3:V45" si="0">V4+U3</f>
         <v>1032008.2166187072</v>
       </c>
@@ -8676,7 +8679,7 @@
         <f>V4/U3</f>
         <v>11.624886524820923</v>
       </c>
-      <c r="X3" s="66">
+      <c r="X3" s="65">
         <f>(G3-W3)/G3</f>
         <v>9.7613057270732931E-6</v>
       </c>
@@ -8727,7 +8730,7 @@
         <f>(1+L$2)^(-(A4-A$3))</f>
         <v>0.96153846153846145</v>
       </c>
-      <c r="Q4" s="63">
+      <c r="Q4" s="62">
         <f>B4*P4/B$3</f>
         <v>0.94805771726540722</v>
       </c>
@@ -8743,11 +8746,11 @@
         <f t="shared" ref="T4:T47" si="6">(1+L$2)^-A4</f>
         <v>9.1404231750869397E-2</v>
       </c>
-      <c r="U4" s="64">
+      <c r="U4" s="63">
         <f t="shared" ref="U4:U48" si="7">T4*J4</f>
         <v>77497.989892149679</v>
       </c>
-      <c r="V4" s="65">
+      <c r="V4" s="64">
         <f t="shared" si="0"/>
         <v>950264.25681441533</v>
       </c>
@@ -8755,7 +8758,7 @@
         <f t="shared" ref="W4:W47" si="8">V5/U4</f>
         <v>11.261792314056835</v>
       </c>
-      <c r="X4" s="66">
+      <c r="X4" s="65">
         <f t="shared" ref="X4:X47" si="9">(G4-W4)/G4</f>
         <v>1.8441302003640874E-5</v>
       </c>
@@ -8803,10 +8806,10 @@
         <v>7.4933920704845836E-2</v>
       </c>
       <c r="P5" s="54">
-        <f t="shared" ref="P5:P48" si="12">(1+L$2)^(-(A5-A$3))</f>
+        <f t="shared" ref="P5:P47" si="12">(1+L$2)^(-(A5-A$3))</f>
         <v>0.92455621301775137</v>
       </c>
-      <c r="Q5" s="63">
+      <c r="Q5" s="62">
         <f t="shared" ref="Q5:Q47" si="13">B5*P5/B$3</f>
         <v>0.89750062555993149</v>
       </c>
@@ -8822,11 +8825,11 @@
         <f t="shared" si="6"/>
         <v>8.7888684375835968E-2</v>
       </c>
-      <c r="U5" s="64">
+      <c r="U5" s="63">
         <f t="shared" si="7"/>
         <v>73365.260546554855</v>
       </c>
-      <c r="V5" s="65">
+      <c r="V5" s="64">
         <f t="shared" si="0"/>
         <v>872766.26692226564</v>
       </c>
@@ -8834,7 +8837,7 @@
         <f t="shared" si="8"/>
         <v>10.896178932922085</v>
       </c>
-      <c r="X5" s="66">
+      <c r="X5" s="65">
         <f t="shared" si="9"/>
         <v>-1.6421890793363146E-5</v>
       </c>
@@ -8885,7 +8888,7 @@
         <f t="shared" si="12"/>
         <v>0.88899635867091487</v>
       </c>
-      <c r="Q6" s="63">
+      <c r="Q6" s="62">
         <f t="shared" si="13"/>
         <v>0.84825877323998033</v>
       </c>
@@ -8901,11 +8904,11 @@
         <f t="shared" si="6"/>
         <v>8.4508350361380741E-2</v>
       </c>
-      <c r="U6" s="64">
+      <c r="U6" s="63">
         <f t="shared" si="7"/>
         <v>69340.047309260219</v>
       </c>
-      <c r="V6" s="65">
+      <c r="V6" s="64">
         <f t="shared" si="0"/>
         <v>799401.00637571083</v>
       </c>
@@ -8913,7 +8916,7 @@
         <f t="shared" si="8"/>
         <v>10.52870581138113</v>
       </c>
-      <c r="X6" s="66">
+      <c r="X6" s="65">
         <f t="shared" si="9"/>
         <v>2.7940793890217004E-5</v>
       </c>
@@ -8964,7 +8967,7 @@
         <f t="shared" si="12"/>
         <v>0.85480419102972571</v>
       </c>
-      <c r="Q7" s="63">
+      <c r="Q7" s="62">
         <f t="shared" si="13"/>
         <v>0.80027527902095319</v>
       </c>
@@ -8980,11 +8983,11 @@
         <f t="shared" si="6"/>
         <v>8.1258029193635312E-2</v>
       </c>
-      <c r="U7" s="64">
+      <c r="U7" s="63">
         <f t="shared" si="7"/>
         <v>65417.667517718117</v>
       </c>
-      <c r="V7" s="65">
+      <c r="V7" s="64">
         <f t="shared" si="0"/>
         <v>730060.9590664506</v>
       </c>
@@ -8992,7 +8995,7 @@
         <f t="shared" si="8"/>
         <v>10.159996783265262</v>
       </c>
-      <c r="X7" s="66">
+      <c r="X7" s="65">
         <f t="shared" si="9"/>
         <v>3.1660774981611975E-7</v>
       </c>
@@ -9043,7 +9046,7 @@
         <f t="shared" si="12"/>
         <v>0.82192710675935154</v>
       </c>
-      <c r="Q8" s="63">
+      <c r="Q8" s="62">
         <f t="shared" si="13"/>
         <v>0.75349021194175358</v>
       </c>
@@ -9059,11 +9062,11 @@
         <f t="shared" si="6"/>
         <v>7.8132720378495488E-2</v>
       </c>
-      <c r="U8" s="64">
+      <c r="U8" s="63">
         <f t="shared" si="7"/>
         <v>61593.250032066891</v>
       </c>
-      <c r="V8" s="65">
+      <c r="V8" s="64">
         <f t="shared" si="0"/>
         <v>664643.29154873244</v>
       </c>
@@ -9071,7 +9074,7 @@
         <f t="shared" si="8"/>
         <v>9.7908462567359837</v>
       </c>
-      <c r="X8" s="66">
+      <c r="X8" s="65">
         <f t="shared" si="9"/>
         <v>1.5702508836342137E-5</v>
       </c>
@@ -9122,7 +9125,7 @@
         <f t="shared" si="12"/>
         <v>0.79031452573014571</v>
       </c>
-      <c r="Q9" s="63">
+      <c r="Q9" s="62">
         <f t="shared" si="13"/>
         <v>0.70786747802525374</v>
       </c>
@@ -9135,11 +9138,11 @@
         <f t="shared" si="6"/>
         <v>7.5127615748553353E-2</v>
       </c>
-      <c r="U9" s="64">
+      <c r="U9" s="63">
         <f t="shared" si="7"/>
         <v>57863.897191182994</v>
       </c>
-      <c r="V9" s="65">
+      <c r="V9" s="64">
         <f t="shared" si="0"/>
         <v>603050.0415166656</v>
       </c>
@@ -9147,7 +9150,7 @@
         <f t="shared" si="8"/>
         <v>9.4218704717413218</v>
       </c>
-      <c r="X9" s="66">
+      <c r="X9" s="65">
         <f t="shared" si="9"/>
         <v>1.3747427157593502E-5</v>
       </c>
@@ -9198,7 +9201,7 @@
         <f t="shared" si="12"/>
         <v>0.75991781320206331</v>
       </c>
-      <c r="Q10" s="63">
+      <c r="Q10" s="62">
         <f t="shared" si="13"/>
         <v>0.663367009868709</v>
       </c>
@@ -9211,11 +9214,11 @@
         <f t="shared" si="6"/>
         <v>7.2238092065916693E-2</v>
       </c>
-      <c r="U10" s="64">
+      <c r="U10" s="63">
         <f t="shared" si="7"/>
         <v>54226.261038914206</v>
       </c>
-      <c r="V10" s="65">
+      <c r="V10" s="64">
         <f t="shared" si="0"/>
         <v>545186.14432548266</v>
       </c>
@@ -9223,7 +9226,7 @@
         <f t="shared" si="8"/>
         <v>9.0539136182419551</v>
       </c>
-      <c r="X10" s="66">
+      <c r="X10" s="65">
         <f t="shared" si="9"/>
         <v>9.5407287436720154E-6</v>
       </c>
@@ -9274,7 +9277,7 @@
         <f t="shared" si="12"/>
         <v>0.73069020500198378</v>
       </c>
-      <c r="Q11" s="63">
+      <c r="Q11" s="62">
         <f t="shared" si="13"/>
         <v>0.61997387731283338</v>
       </c>
@@ -9287,11 +9290,11 @@
         <f t="shared" si="6"/>
         <v>6.9459703909535264E-2</v>
       </c>
-      <c r="U11" s="64">
+      <c r="U11" s="63">
         <f t="shared" si="7"/>
         <v>50679.133598070606</v>
       </c>
-      <c r="V11" s="65">
+      <c r="V11" s="64">
         <f t="shared" si="0"/>
         <v>490959.88328656845</v>
       </c>
@@ -9299,7 +9302,7 @@
         <f t="shared" si="8"/>
         <v>8.6876139829126782</v>
       </c>
-      <c r="X11" s="66">
+      <c r="X11" s="65">
         <f t="shared" si="9"/>
         <v>4.4431064378734266E-5</v>
       </c>
@@ -9350,7 +9353,7 @@
         <f t="shared" si="12"/>
         <v>0.70258673557883045</v>
       </c>
-      <c r="Q12" s="63">
+      <c r="Q12" s="62">
         <f t="shared" si="13"/>
         <v>0.57767258622505047</v>
       </c>
@@ -9363,11 +9366,11 @@
         <f t="shared" si="6"/>
         <v>6.6788176836091603E-2</v>
       </c>
-      <c r="U12" s="64">
+      <c r="U12" s="63">
         <f t="shared" si="7"/>
         <v>47221.257328725333</v>
       </c>
-      <c r="V12" s="65">
+      <c r="V12" s="64">
         <f t="shared" si="0"/>
         <v>440280.74968849786</v>
       </c>
@@ -9375,7 +9378,7 @@
         <f t="shared" si="8"/>
         <v>8.3237828595611987</v>
       </c>
-      <c r="X12" s="66">
+      <c r="X12" s="65">
         <f t="shared" si="9"/>
         <v>2.6086069053479894E-5</v>
       </c>
@@ -9426,7 +9429,7 @@
         <f t="shared" si="12"/>
         <v>0.67556416882579851</v>
       </c>
-      <c r="Q13" s="63">
+      <c r="Q13" s="62">
         <f t="shared" si="13"/>
         <v>0.5364582036881469</v>
       </c>
@@ -9439,11 +9442,11 @@
         <f t="shared" si="6"/>
         <v>6.4219400803934235E-2</v>
       </c>
-      <c r="U13" s="64">
+      <c r="U13" s="63">
         <f t="shared" si="7"/>
         <v>43852.202238541278</v>
       </c>
-      <c r="V13" s="65">
+      <c r="V13" s="64">
         <f t="shared" si="0"/>
         <v>393059.49235977256</v>
       </c>
@@ -9451,7 +9454,7 @@
         <f t="shared" si="8"/>
         <v>7.9632782915134044</v>
       </c>
-      <c r="X13" s="66">
+      <c r="X13" s="65">
         <f t="shared" si="9"/>
         <v>-3.4948074017870797E-5</v>
       </c>
@@ -9502,7 +9505,7 @@
         <f t="shared" si="12"/>
         <v>0.6495809315632679</v>
       </c>
-      <c r="Q14" s="63">
+      <c r="Q14" s="62">
         <f t="shared" si="13"/>
         <v>0.49634795070512722</v>
       </c>
@@ -9515,11 +9518,11 @@
         <f t="shared" si="6"/>
         <v>6.1749423849936765E-2</v>
       </c>
-      <c r="U14" s="64">
+      <c r="U14" s="63">
         <f t="shared" si="7"/>
         <v>40573.40680962881</v>
       </c>
-      <c r="V14" s="65">
+      <c r="V14" s="64">
         <f t="shared" si="0"/>
         <v>349207.29012123129</v>
       </c>
@@ -9527,7 +9530,7 @@
         <f t="shared" si="8"/>
         <v>7.6068022771594821</v>
       </c>
-      <c r="X14" s="66">
+      <c r="X14" s="65">
         <f t="shared" si="9"/>
         <v>2.5992223020653456E-5</v>
       </c>
@@ -9578,7 +9581,7 @@
         <f t="shared" si="12"/>
         <v>0.62459704958006512</v>
       </c>
-      <c r="Q15" s="63">
+      <c r="Q15" s="62">
         <f t="shared" si="13"/>
         <v>0.45735574849273802</v>
       </c>
@@ -9591,11 +9594,11 @@
         <f t="shared" si="6"/>
         <v>5.937444600955457E-2</v>
       </c>
-      <c r="U15" s="64">
+      <c r="U15" s="63">
         <f t="shared" si="7"/>
         <v>37386.053601603155</v>
       </c>
-      <c r="V15" s="65">
+      <c r="V15" s="64">
         <f t="shared" si="0"/>
         <v>308633.88331160246</v>
       </c>
@@ -9603,7 +9606,7 @@
         <f t="shared" si="8"/>
         <v>7.2553212649962049</v>
       </c>
-      <c r="X15" s="66">
+      <c r="X15" s="65">
         <f t="shared" si="9"/>
         <v>-4.4281874046174384E-5</v>
       </c>
@@ -9654,7 +9657,7 @@
         <f t="shared" si="12"/>
         <v>0.600574086134678</v>
       </c>
-      <c r="Q16" s="63">
+      <c r="Q16" s="62">
         <f t="shared" si="13"/>
         <v>0.41952731107009711</v>
       </c>
@@ -9667,11 +9670,11 @@
         <f t="shared" si="6"/>
         <v>5.7090813470725546E-2</v>
       </c>
-      <c r="U16" s="64">
+      <c r="U16" s="63">
         <f t="shared" si="7"/>
         <v>34293.795591209018</v>
       </c>
-      <c r="V16" s="65">
+      <c r="V16" s="64">
         <f t="shared" si="0"/>
         <v>271247.82970999932</v>
       </c>
@@ -9679,7 +9682,7 @@
         <f t="shared" si="8"/>
         <v>6.9095307192981545</v>
       </c>
-      <c r="X16" s="66">
+      <c r="X16" s="65">
         <f t="shared" si="9"/>
         <v>6.7913270889377429E-5</v>
       </c>
@@ -9730,7 +9733,7 @@
         <f t="shared" si="12"/>
         <v>0.57747508282180582</v>
       </c>
-      <c r="Q17" s="63">
+      <c r="Q17" s="62">
         <f t="shared" si="13"/>
         <v>0.38291949693379929</v>
       </c>
@@ -9743,11 +9746,11 @@
         <f t="shared" si="6"/>
         <v>5.4895012952620711E-2</v>
       </c>
-      <c r="U17" s="64">
+      <c r="U17" s="63">
         <f t="shared" si="7"/>
         <v>31301.332177841501</v>
       </c>
-      <c r="V17" s="65">
+      <c r="V17" s="64">
         <f t="shared" si="0"/>
         <v>236954.03411879033</v>
       </c>
@@ -9755,7 +9758,7 @@
         <f t="shared" si="8"/>
         <v>6.570094230255549</v>
       </c>
-      <c r="X17" s="66">
+      <c r="X17" s="65">
         <f t="shared" si="9"/>
         <v>-1.4342504649720893E-5</v>
       </c>
@@ -9806,7 +9809,7 @@
         <f t="shared" si="12"/>
         <v>0.55526450271327477</v>
       </c>
-      <c r="Q18" s="63">
+      <c r="Q18" s="62">
         <f t="shared" si="13"/>
         <v>0.34759143576239832</v>
       </c>
@@ -9819,11 +9822,11 @@
         <f t="shared" si="6"/>
         <v>5.2783666300596846E-2</v>
       </c>
-      <c r="U18" s="64">
+      <c r="U18" s="63">
         <f t="shared" si="7"/>
         <v>28413.483310087762</v>
       </c>
-      <c r="V18" s="65">
+      <c r="V18" s="64">
         <f t="shared" si="0"/>
         <v>205652.70194094881</v>
       </c>
@@ -9831,7 +9834,7 @@
         <f t="shared" si="8"/>
         <v>6.2378560451943974</v>
       </c>
-      <c r="X18" s="66">
+      <c r="X18" s="65">
         <f t="shared" si="9"/>
         <v>2.3077076884102342E-5</v>
       </c>
@@ -9882,7 +9885,7 @@
         <f t="shared" si="12"/>
         <v>0.53390817568584104</v>
       </c>
-      <c r="Q19" s="63">
+      <c r="Q19" s="62">
         <f t="shared" si="13"/>
         <v>0.31362097891239615</v>
       </c>
@@ -9895,11 +9898,11 @@
         <f t="shared" si="6"/>
         <v>5.0753525289035421E-2</v>
       </c>
-      <c r="U19" s="64">
+      <c r="U19" s="63">
         <f t="shared" si="7"/>
         <v>25636.611729667256</v>
       </c>
-      <c r="V19" s="65">
+      <c r="V19" s="64">
         <f t="shared" si="0"/>
         <v>177239.21863086105</v>
       </c>
@@ -9907,7 +9910,7 @@
         <f t="shared" si="8"/>
         <v>5.9135196374548942</v>
       </c>
-      <c r="X19" s="66">
+      <c r="X19" s="65">
         <f t="shared" si="9"/>
         <v>8.1224644082774481E-5</v>
       </c>
@@ -9958,7 +9961,7 @@
         <f t="shared" si="12"/>
         <v>0.51337324585177024</v>
       </c>
-      <c r="Q20" s="63">
+      <c r="Q20" s="62">
         <f t="shared" si="13"/>
         <v>0.28109512928772701</v>
       </c>
@@ -9971,11 +9974,11 @@
         <f t="shared" si="6"/>
         <v>4.8801466624072518E-2</v>
       </c>
-      <c r="U20" s="64">
+      <c r="U20" s="63">
         <f t="shared" si="7"/>
         <v>22977.799286242342</v>
       </c>
-      <c r="V20" s="65">
+      <c r="V20" s="64">
         <f t="shared" si="0"/>
         <v>151602.60690119379</v>
       </c>
@@ -9983,7 +9986,7 @@
         <f t="shared" si="8"/>
         <v>5.5977861940836036</v>
       </c>
-      <c r="X20" s="66">
+      <c r="X20" s="65">
         <f t="shared" si="9"/>
         <v>3.8193268380904528E-5</v>
       </c>
@@ -10034,7 +10037,7 @@
         <f t="shared" si="12"/>
         <v>0.49362812101131748</v>
       </c>
-      <c r="Q21" s="63">
+      <c r="Q21" s="62">
         <f t="shared" si="13"/>
         <v>0.25011250731131301</v>
       </c>
@@ -10047,11 +10050,11 @@
         <f t="shared" si="6"/>
         <v>4.6924487138531264E-2</v>
       </c>
-      <c r="U21" s="64">
+      <c r="U21" s="63">
         <f t="shared" si="7"/>
         <v>20445.159736067377</v>
       </c>
-      <c r="V21" s="65">
+      <c r="V21" s="64">
         <f t="shared" si="0"/>
         <v>128624.80761495145</v>
       </c>
@@ -10059,7 +10062,7 @@
         <f t="shared" si="8"/>
         <v>5.2912106960966403</v>
       </c>
-      <c r="X21" s="66">
+      <c r="X21" s="65">
         <f t="shared" si="9"/>
         <v>-3.982160208654857E-5</v>
       </c>
@@ -10110,7 +10113,7 @@
         <f t="shared" si="12"/>
         <v>0.47464242404934376</v>
       </c>
-      <c r="Q22" s="63">
+      <c r="Q22" s="62">
         <f t="shared" si="13"/>
         <v>0.22077499594574421</v>
       </c>
@@ -10123,11 +10126,11 @@
         <f t="shared" si="6"/>
         <v>4.5119699171664682E-2</v>
       </c>
-      <c r="U22" s="64">
+      <c r="U22" s="63">
         <f t="shared" si="7"/>
         <v>18046.981816641553</v>
       </c>
-      <c r="V22" s="65">
+      <c r="V22" s="64">
         <f t="shared" si="0"/>
         <v>108179.64787888408</v>
       </c>
@@ -10135,7 +10138,7 @@
         <f t="shared" si="8"/>
         <v>4.9943346193837819</v>
       </c>
-      <c r="X22" s="66">
+      <c r="X22" s="65">
         <f t="shared" si="9"/>
         <v>-6.700428189469316E-5</v>
       </c>
@@ -10186,7 +10189,7 @@
         <f t="shared" si="12"/>
         <v>0.45638694620129205</v>
       </c>
-      <c r="Q23" s="63">
+      <c r="Q23" s="62">
         <f t="shared" si="13"/>
         <v>0.19318252124016125</v>
       </c>
@@ -10199,11 +10202,11 @@
         <f t="shared" si="6"/>
         <v>4.3384326126600647E-2</v>
       </c>
-      <c r="U23" s="64">
+      <c r="U23" s="63">
         <f t="shared" si="7"/>
         <v>15791.456146903985</v>
       </c>
-      <c r="V23" s="65">
+      <c r="V23" s="64">
         <f t="shared" si="0"/>
         <v>90132.666062242526</v>
       </c>
@@ -10211,7 +10214,7 @@
         <f t="shared" si="8"/>
         <v>4.7076855499430046</v>
       </c>
-      <c r="X23" s="66">
+      <c r="X23" s="65">
         <f t="shared" si="9"/>
         <v>6.6790581349956797E-5</v>
       </c>
@@ -10262,7 +10265,7 @@
         <f t="shared" si="12"/>
         <v>0.43883360211662686</v>
       </c>
-      <c r="Q24" s="63">
+      <c r="Q24" s="62">
         <f t="shared" si="13"/>
         <v>0.16743545554130992</v>
       </c>
@@ -10275,11 +10278,11 @@
         <f t="shared" si="6"/>
         <v>4.171569819865447E-2</v>
       </c>
-      <c r="U24" s="64">
+      <c r="U24" s="63">
         <f t="shared" si="7"/>
         <v>13686.789092555564</v>
       </c>
-      <c r="V24" s="65">
+      <c r="V24" s="64">
         <f t="shared" si="0"/>
         <v>74341.209915338535</v>
       </c>
@@ -10287,7 +10290,7 @@
         <f t="shared" si="8"/>
         <v>4.4316033813784532</v>
       </c>
-      <c r="X24" s="66">
+      <c r="X24" s="65">
         <f t="shared" si="9"/>
         <v>8.9489761179413875E-5</v>
       </c>
@@ -10338,7 +10341,7 @@
         <f t="shared" si="12"/>
         <v>0.42195538665060278</v>
       </c>
-      <c r="Q25" s="63">
+      <c r="Q25" s="62">
         <f t="shared" si="13"/>
         <v>0.14361623991750175</v>
       </c>
@@ -10351,11 +10354,11 @@
         <f t="shared" si="6"/>
         <v>4.0111248267936987E-2</v>
       </c>
-      <c r="U25" s="64">
+      <c r="U25" s="63">
         <f t="shared" si="7"/>
         <v>11739.711740398257</v>
       </c>
-      <c r="V25" s="65">
+      <c r="V25" s="64">
         <f t="shared" si="0"/>
         <v>60654.420822782966</v>
       </c>
@@ -10363,7 +10366,7 @@
         <f t="shared" si="8"/>
         <v>4.16660222704287</v>
       </c>
-      <c r="X25" s="66">
+      <c r="X25" s="65">
         <f t="shared" si="9"/>
         <v>9.5457873081314688E-5</v>
       </c>
@@ -10414,7 +10417,7 @@
         <f t="shared" si="12"/>
         <v>0.40572633331788732</v>
       </c>
-      <c r="Q26" s="63">
+      <c r="Q26" s="62">
         <f t="shared" si="13"/>
         <v>0.12180056301547199</v>
       </c>
@@ -10427,11 +10430,11 @@
         <f t="shared" si="6"/>
         <v>3.8568507949939407E-2</v>
       </c>
-      <c r="U26" s="64">
+      <c r="U26" s="63">
         <f t="shared" si="7"/>
         <v>9956.4043742942995</v>
       </c>
-      <c r="V26" s="65">
+      <c r="V26" s="64">
         <f t="shared" si="0"/>
         <v>48914.70908238471</v>
       </c>
@@ -10439,7 +10442,7 @@
         <f t="shared" si="8"/>
         <v>3.912888955040231</v>
       </c>
-      <c r="X26" s="66">
+      <c r="X26" s="65">
         <f t="shared" si="9"/>
         <v>2.8378471701704333E-5</v>
       </c>
@@ -10490,7 +10493,7 @@
         <f t="shared" si="12"/>
         <v>0.39012147434412242</v>
       </c>
-      <c r="Q27" s="63">
+      <c r="Q27" s="62">
         <f t="shared" si="13"/>
         <v>0.10203852646489034</v>
       </c>
@@ -10503,11 +10506,11 @@
         <f t="shared" si="6"/>
         <v>3.7085103798018659E-2</v>
       </c>
-      <c r="U27" s="64">
+      <c r="U27" s="63">
         <f t="shared" si="7"/>
         <v>8340.9777645650502</v>
       </c>
-      <c r="V27" s="65">
+      <c r="V27" s="64">
         <f t="shared" si="0"/>
         <v>38958.304708090407</v>
       </c>
@@ -10515,7 +10518,7 @@
         <f t="shared" si="8"/>
         <v>3.6707119725935309</v>
       </c>
-      <c r="X27" s="66">
+      <c r="X27" s="65">
         <f t="shared" si="9"/>
         <v>7.8460203342124244E-5</v>
       </c>
@@ -10566,7 +10569,7 @@
         <f t="shared" si="12"/>
         <v>0.37511680225396377</v>
       </c>
-      <c r="Q28" s="63">
+      <c r="Q28" s="62">
         <f t="shared" si="13"/>
         <v>8.4355433266345189E-2</v>
       </c>
@@ -10579,11 +10582,11 @@
         <f t="shared" si="6"/>
         <v>3.5658753651941009E-2</v>
       </c>
-      <c r="U28" s="64">
+      <c r="U28" s="63">
         <f t="shared" si="7"/>
         <v>6895.50235830778</v>
       </c>
-      <c r="V28" s="65">
+      <c r="V28" s="64">
         <f t="shared" si="0"/>
         <v>30617.326943525353</v>
       </c>
@@ -10591,7 +10594,7 @@
         <f t="shared" si="8"/>
         <v>3.4401880171409482</v>
       </c>
-      <c r="X28" s="66">
+      <c r="X28" s="65">
         <f t="shared" si="9"/>
         <v>-5.4656145624503883E-5</v>
       </c>
@@ -10642,7 +10645,7 @@
         <f t="shared" si="12"/>
         <v>0.36068923293650368</v>
       </c>
-      <c r="Q29" s="63">
+      <c r="Q29" s="62">
         <f t="shared" si="13"/>
         <v>6.8744855477622616E-2</v>
       </c>
@@ -10655,11 +10658,11 @@
         <f t="shared" si="6"/>
         <v>3.4287263126866356E-2</v>
       </c>
-      <c r="U29" s="64">
+      <c r="U29" s="63">
         <f t="shared" si="7"/>
         <v>5619.4366045770912</v>
       </c>
-      <c r="V29" s="65">
+      <c r="V29" s="64">
         <f t="shared" si="0"/>
         <v>23721.824585217575</v>
       </c>
@@ -10667,7 +10670,7 @@
         <f t="shared" si="8"/>
         <v>3.2213884156813686</v>
       </c>
-      <c r="X29" s="66">
+      <c r="X29" s="65">
         <f t="shared" si="9"/>
         <v>1.8981512061806252E-4</v>
       </c>
@@ -10718,7 +10721,7 @@
         <f t="shared" si="12"/>
         <v>0.3468165701312535</v>
       </c>
-      <c r="Q30" s="63">
+      <c r="Q30" s="62">
         <f t="shared" si="13"/>
         <v>5.5166967155900554E-2</v>
       </c>
@@ -10731,11 +10734,11 @@
         <f t="shared" si="6"/>
         <v>3.2968522237371505E-2</v>
       </c>
-      <c r="U30" s="64">
+      <c r="U30" s="63">
         <f t="shared" si="7"/>
         <v>4509.5438421288418</v>
       </c>
-      <c r="V30" s="65">
+      <c r="V30" s="64">
         <f t="shared" si="0"/>
         <v>18102.387980640484</v>
       </c>
@@ -10743,7 +10746,7 @@
         <f t="shared" si="8"/>
         <v>3.0142392699512603</v>
       </c>
-      <c r="X30" s="66">
+      <c r="X30" s="65">
         <f t="shared" si="9"/>
         <v>2.5231510737637718E-4</v>
       </c>
@@ -10794,7 +10797,7 @@
         <f t="shared" si="12"/>
         <v>0.3334774712800514</v>
       </c>
-      <c r="Q31" s="63">
+      <c r="Q31" s="62">
         <f t="shared" si="13"/>
         <v>4.3544778025006919E-2</v>
       </c>
@@ -10807,11 +10810,11 @@
         <f t="shared" si="6"/>
         <v>3.1700502151318748E-2</v>
       </c>
-      <c r="U31" s="64">
+      <c r="U31" s="63">
         <f t="shared" si="7"/>
         <v>3559.5043653880439</v>
       </c>
-      <c r="V31" s="65">
+      <c r="V31" s="64">
         <f t="shared" si="0"/>
         <v>13592.844138511642</v>
       </c>
@@ -10819,7 +10822,7 @@
         <f t="shared" si="8"/>
         <v>2.8187463037511407</v>
       </c>
-      <c r="X31" s="66">
+      <c r="X31" s="65">
         <f t="shared" si="9"/>
         <v>8.9995121979174165E-5</v>
       </c>
@@ -10870,7 +10873,7 @@
         <f t="shared" si="12"/>
         <v>0.32065141469235708</v>
       </c>
-      <c r="Q32" s="63">
+      <c r="Q32" s="62">
         <f t="shared" si="13"/>
         <v>3.3769756660864472E-2</v>
       </c>
@@ -10883,11 +10886,11 @@
         <f t="shared" si="6"/>
         <v>3.0481252068575718E-2</v>
       </c>
-      <c r="U32" s="64">
+      <c r="U32" s="63">
         <f t="shared" si="7"/>
         <v>2760.4640873654548</v>
       </c>
-      <c r="V32" s="65">
+      <c r="V32" s="64">
         <f t="shared" si="0"/>
         <v>10033.339773123598</v>
       </c>
@@ -10895,7 +10898,7 @@
         <f>V33/U32</f>
         <v>2.6346568749239792</v>
       </c>
-      <c r="X32" s="66">
+      <c r="X32" s="65">
         <f t="shared" si="9"/>
         <v>1.3021824516912104E-4</v>
       </c>
@@ -10946,7 +10949,7 @@
         <f t="shared" si="12"/>
         <v>0.30831866797342034</v>
       </c>
-      <c r="Q33" s="63">
+      <c r="Q33" s="62">
         <f t="shared" si="13"/>
         <v>2.5701229838345507E-2</v>
       </c>
@@ -10959,11 +10962,11 @@
         <f t="shared" si="6"/>
         <v>2.9308896219784344E-2</v>
       </c>
-      <c r="U33" s="64">
+      <c r="U33" s="63">
         <f t="shared" si="7"/>
         <v>2100.8989709525295</v>
       </c>
-      <c r="V33" s="65">
+      <c r="V33" s="64">
         <f t="shared" si="0"/>
         <v>7272.8756857581438</v>
       </c>
@@ -10971,7 +10974,7 @@
         <f t="shared" si="8"/>
         <v>2.4617922072000846</v>
       </c>
-      <c r="X33" s="66">
+      <c r="X33" s="65">
         <f t="shared" si="9"/>
         <v>4.9037466500830387E-4</v>
       </c>
@@ -11022,7 +11025,7 @@
         <f t="shared" si="12"/>
         <v>0.29646025766675027</v>
       </c>
-      <c r="Q34" s="63">
+      <c r="Q34" s="62">
         <f t="shared" si="13"/>
         <v>1.9173888717495643E-2</v>
       </c>
@@ -11035,11 +11038,11 @@
         <f t="shared" si="6"/>
         <v>2.8181630980561867E-2</v>
       </c>
-      <c r="U34" s="64">
+      <c r="U34" s="63">
         <f t="shared" si="7"/>
         <v>1567.3312351855184</v>
       </c>
-      <c r="V34" s="65">
+      <c r="V34" s="64">
         <f t="shared" si="0"/>
         <v>5171.9767148056144</v>
       </c>
@@ -11047,7 +11050,7 @@
         <f t="shared" si="8"/>
         <v>2.2998619555957673</v>
       </c>
-      <c r="X34" s="66">
+      <c r="X34" s="65">
         <f t="shared" si="9"/>
         <v>4.9458687711117708E-4</v>
       </c>
@@ -11098,7 +11101,7 @@
         <f t="shared" si="12"/>
         <v>0.28505794006418295</v>
       </c>
-      <c r="Q35" s="63">
+      <c r="Q35" s="62">
         <f t="shared" si="13"/>
         <v>1.400566795793046E-2</v>
       </c>
@@ -11111,11 +11114,11 @@
         <f t="shared" si="6"/>
         <v>2.7097722096694102E-2</v>
       </c>
-      <c r="U35" s="64">
+      <c r="U35" s="63">
         <f t="shared" si="7"/>
         <v>1144.8751853324372</v>
       </c>
-      <c r="V35" s="65">
+      <c r="V35" s="64">
         <f t="shared" si="0"/>
         <v>3604.645479620096</v>
       </c>
@@ -11123,7 +11126,7 @@
         <f t="shared" si="8"/>
         <v>2.1485052045856126</v>
       </c>
-      <c r="X35" s="66">
+      <c r="X35" s="65">
         <f t="shared" si="9"/>
         <v>6.9525368111039579E-4</v>
       </c>
@@ -11174,7 +11177,7 @@
         <f t="shared" si="12"/>
         <v>0.27409417313863743</v>
       </c>
-      <c r="Q36" s="63">
+      <c r="Q36" s="62">
         <f t="shared" si="13"/>
         <v>1.0006052083189644E-2</v>
       </c>
@@ -11187,11 +11190,11 @@
         <f t="shared" si="6"/>
         <v>2.6055502016052019E-2</v>
       </c>
-      <c r="U36" s="64">
+      <c r="U36" s="63">
         <f t="shared" si="7"/>
         <v>817.9362610133212</v>
       </c>
-      <c r="V36" s="65">
+      <c r="V36" s="64">
         <f t="shared" si="0"/>
         <v>2459.770294287659</v>
       </c>
@@ -11199,7 +11202,7 @@
         <f t="shared" si="8"/>
         <v>2.0072884789828365</v>
       </c>
-      <c r="X36" s="66">
+      <c r="X36" s="65">
         <f t="shared" si="9"/>
         <v>8.5192683781156354E-4</v>
       </c>
@@ -11250,7 +11253,7 @@
         <f t="shared" si="12"/>
         <v>0.26355208955638215</v>
       </c>
-      <c r="Q37" s="63">
+      <c r="Q37" s="62">
         <f t="shared" si="13"/>
         <v>6.9845061249010285E-3</v>
       </c>
@@ -11263,11 +11266,11 @@
         <f t="shared" si="6"/>
         <v>2.5053367323126945E-2</v>
       </c>
-      <c r="U37" s="64">
+      <c r="U37" s="63">
         <f t="shared" si="7"/>
         <v>570.94310450251976</v>
       </c>
-      <c r="V37" s="65">
+      <c r="V37" s="64">
         <f t="shared" si="0"/>
         <v>1641.8340332743378</v>
       </c>
@@ -11275,7 +11278,7 @@
         <f t="shared" si="8"/>
         <v>1.8756526181447064</v>
       </c>
-      <c r="X37" s="66">
+      <c r="X37" s="65">
         <f t="shared" si="9"/>
         <v>1.7814698538018076E-3</v>
       </c>
@@ -11326,7 +11329,7 @@
         <f t="shared" si="12"/>
         <v>0.25341547072729048</v>
       </c>
-      <c r="Q38" s="63">
+      <c r="Q38" s="62">
         <f t="shared" si="13"/>
         <v>4.7587822779251538E-3</v>
       </c>
@@ -11339,11 +11342,11 @@
         <f t="shared" si="6"/>
         <v>2.4089776272237445E-2</v>
       </c>
-      <c r="U38" s="64">
+      <c r="U38" s="63">
         <f t="shared" si="7"/>
         <v>388.99341880514459</v>
       </c>
-      <c r="V38" s="65">
+      <c r="V38" s="64">
         <f t="shared" si="0"/>
         <v>1070.8909287718179</v>
       </c>
@@ -11351,7 +11354,7 @@
         <f t="shared" si="8"/>
         <v>1.7529795544131068</v>
       </c>
-      <c r="X38" s="66">
+      <c r="X38" s="65">
         <f t="shared" si="9"/>
         <v>2.2882445002237184E-3</v>
       </c>
@@ -11402,7 +11405,7 @@
         <f t="shared" si="12"/>
         <v>0.24366872185316396</v>
       </c>
-      <c r="Q39" s="63">
+      <c r="Q39" s="62">
         <f t="shared" si="13"/>
         <v>3.1617688221147223E-3</v>
       </c>
@@ -11415,11 +11418,11 @@
         <f t="shared" si="6"/>
         <v>2.3163246415612924E-2</v>
       </c>
-      <c r="U39" s="64">
+      <c r="U39" s="63">
         <f t="shared" si="7"/>
         <v>258.4449832613372</v>
       </c>
-      <c r="V39" s="65">
+      <c r="V39" s="64">
         <f t="shared" si="0"/>
         <v>681.8975099666734</v>
       </c>
@@ -11427,7 +11430,7 @@
         <f t="shared" si="8"/>
         <v>1.6384629384627862</v>
       </c>
-      <c r="X39" s="66">
+      <c r="X39" s="65">
         <f t="shared" si="9"/>
         <v>3.9738975910114192E-3</v>
       </c>
@@ -11478,7 +11481,7 @@
         <f t="shared" si="12"/>
         <v>0.23429684793573452</v>
       </c>
-      <c r="Q40" s="63">
+      <c r="Q40" s="62">
         <f t="shared" si="13"/>
         <v>2.0467556385661361E-3</v>
       </c>
@@ -11491,11 +11494,11 @@
         <f t="shared" si="6"/>
         <v>2.2272352322704737E-2</v>
       </c>
-      <c r="U40" s="64">
+      <c r="U40" s="63">
         <f t="shared" si="7"/>
         <v>167.3108210388082</v>
       </c>
-      <c r="V40" s="65">
+      <c r="V40" s="64">
         <f t="shared" si="0"/>
         <v>423.45252670533614</v>
       </c>
@@ -11503,7 +11506,7 @@
         <f t="shared" si="8"/>
         <v>1.5309332897668055</v>
       </c>
-      <c r="X40" s="66">
+      <c r="X40" s="65">
         <f t="shared" si="9"/>
         <v>6.5325828898081684E-3</v>
       </c>
@@ -11554,7 +11557,7 @@
         <f t="shared" si="12"/>
         <v>0.22528543070743706</v>
       </c>
-      <c r="Q41" s="63">
+      <c r="Q41" s="62">
         <f t="shared" si="13"/>
         <v>1.290016072271501E-3</v>
       </c>
@@ -11567,11 +11570,11 @@
         <f t="shared" si="6"/>
         <v>2.141572338721609E-2</v>
       </c>
-      <c r="U41" s="64">
+      <c r="U41" s="63">
         <f t="shared" si="7"/>
         <v>105.46212378076029</v>
       </c>
-      <c r="V41" s="65">
+      <c r="V41" s="64">
         <f t="shared" si="0"/>
         <v>256.14170566652791</v>
       </c>
@@ -11579,7 +11582,7 @@
         <f t="shared" si="8"/>
         <v>1.4287554288116513</v>
       </c>
-      <c r="X41" s="66">
+      <c r="X41" s="65">
         <f t="shared" si="9"/>
         <v>1.0557182263399346E-2</v>
       </c>
@@ -11630,7 +11633,7 @@
         <f t="shared" si="12"/>
         <v>0.21662060644945874</v>
       </c>
-      <c r="Q42" s="63">
+      <c r="Q42" s="62">
         <f t="shared" si="13"/>
         <v>7.9124626691182609E-4</v>
       </c>
@@ -11643,11 +11646,11 @@
         <f t="shared" si="6"/>
         <v>2.0592041718477009E-2</v>
       </c>
-      <c r="U42" s="64">
+      <c r="U42" s="63">
         <f t="shared" si="7"/>
         <v>64.687830174023844</v>
       </c>
-      <c r="V42" s="65">
+      <c r="V42" s="64">
         <f t="shared" si="0"/>
         <v>150.67958188576762</v>
       </c>
@@ -11655,7 +11658,7 @@
         <f t="shared" si="8"/>
         <v>1.3293343041559424</v>
       </c>
-      <c r="X42" s="66">
+      <c r="X42" s="65">
         <f t="shared" si="9"/>
         <v>1.8941472947643936E-2</v>
       </c>
@@ -11706,7 +11709,7 @@
         <f t="shared" si="12"/>
         <v>0.20828904466294101</v>
       </c>
-      <c r="Q43" s="63">
+      <c r="Q43" s="62">
         <f t="shared" si="13"/>
         <v>4.7208721322556161E-4</v>
       </c>
@@ -11719,11 +11722,11 @@
         <f t="shared" si="6"/>
         <v>1.9800040113920201E-2</v>
       </c>
-      <c r="U43" s="64">
+      <c r="U43" s="63">
         <f t="shared" si="7"/>
         <v>38.593754679209916</v>
       </c>
-      <c r="V43" s="65">
+      <c r="V43" s="64">
         <f t="shared" si="0"/>
         <v>85.99175171174376</v>
       </c>
@@ -11731,7 +11734,7 @@
         <f t="shared" si="8"/>
         <v>1.2281260899983564</v>
       </c>
-      <c r="X43" s="66">
+      <c r="X43" s="65">
         <f t="shared" si="9"/>
         <v>3.373242329004212E-2</v>
       </c>
@@ -11782,7 +11785,7 @@
         <f t="shared" si="12"/>
         <v>0.20027792756052021</v>
       </c>
-      <c r="Q44" s="63">
+      <c r="Q44" s="62">
         <f t="shared" si="13"/>
         <v>2.7389517442537618E-4</v>
       </c>
@@ -11795,11 +11798,11 @@
         <f t="shared" si="6"/>
         <v>1.9038500109538652E-2</v>
       </c>
-      <c r="U44" s="64">
+      <c r="U44" s="63">
         <f t="shared" si="7"/>
         <v>22.388830839481656</v>
       </c>
-      <c r="V44" s="65">
+      <c r="V44" s="64">
         <f t="shared" si="0"/>
         <v>47.397997032533844</v>
       </c>
@@ -11807,7 +11810,7 @@
         <f t="shared" si="8"/>
         <v>1.1170376145300849</v>
       </c>
-      <c r="X44" s="66">
+      <c r="X44" s="65">
         <f t="shared" si="9"/>
         <v>6.131292896631519E-2</v>
       </c>
@@ -11858,7 +11861,7 @@
         <f t="shared" si="12"/>
         <v>0.19257493034665407</v>
       </c>
-      <c r="Q45" s="63">
+      <c r="Q45" s="62">
         <f t="shared" si="13"/>
         <v>1.5429893967415964E-4</v>
       </c>
@@ -11871,11 +11874,11 @@
         <f t="shared" si="6"/>
         <v>1.8306250105325626E-2</v>
       </c>
-      <c r="U45" s="64">
+      <c r="U45" s="63">
         <f t="shared" si="7"/>
         <v>12.615245069169472</v>
       </c>
-      <c r="V45" s="65">
+      <c r="V45" s="64">
         <f t="shared" si="0"/>
         <v>25.009166193052188</v>
       </c>
@@ -11883,7 +11886,7 @@
         <f t="shared" si="8"/>
         <v>0.98245583466090158</v>
       </c>
-      <c r="X45" s="66">
+      <c r="X45" s="65">
         <f t="shared" si="9"/>
         <v>0.11729035520134627</v>
       </c>
@@ -11904,7 +11907,7 @@
       <c r="G46" s="5">
         <v>1.0369999999999999</v>
       </c>
-      <c r="H46" s="67" t="s">
+      <c r="H46" s="66" t="s">
         <v>51</v>
       </c>
       <c r="I46" s="6"/>
@@ -11936,7 +11939,7 @@
         <f t="shared" si="12"/>
         <v>0.18516820225639813</v>
       </c>
-      <c r="Q46" s="63">
+      <c r="Q46" s="62">
         <f t="shared" si="13"/>
         <v>8.4195162181249864E-5</v>
       </c>
@@ -11949,11 +11952,11 @@
         <f t="shared" si="6"/>
         <v>1.7602163562813106E-2</v>
       </c>
-      <c r="U46" s="64">
+      <c r="U46" s="63">
         <f t="shared" si="7"/>
         <v>6.8898646147002527</v>
       </c>
-      <c r="V46" s="65">
+      <c r="V46" s="64">
         <f>V47+U46</f>
         <v>12.393921123882716</v>
       </c>
@@ -11961,7 +11964,7 @@
         <f t="shared" si="8"/>
         <v>0.79886279585798792</v>
       </c>
-      <c r="X46" s="66">
+      <c r="X46" s="65">
         <f t="shared" si="9"/>
         <v>0.22964050544070591</v>
       </c>
@@ -12014,7 +12017,7 @@
         <f t="shared" si="12"/>
         <v>0.17804634832345972</v>
       </c>
-      <c r="Q47" s="63">
+      <c r="Q47" s="62">
         <f t="shared" si="13"/>
         <v>4.4515935148949247E-5</v>
       </c>
@@ -12027,11 +12030,11 @@
         <f t="shared" si="6"/>
         <v>1.6925157271935672E-2</v>
       </c>
-      <c r="U47" s="64">
+      <c r="U47" s="63">
         <f t="shared" si="7"/>
         <v>3.64367840200494</v>
       </c>
-      <c r="V47" s="64">
+      <c r="V47" s="63">
         <f>U47+V48</f>
         <v>5.5040565091824627</v>
       </c>
@@ -12039,7 +12042,7 @@
         <f t="shared" si="8"/>
         <v>0.51057692307692326</v>
       </c>
-      <c r="X47" s="66">
+      <c r="X47" s="65">
         <f t="shared" si="9"/>
         <v>0.46870247338509546</v>
       </c>
@@ -12073,11 +12076,11 @@
         <f>(1+L$2)^-A48</f>
         <v>1.6274189684553533E-2</v>
       </c>
-      <c r="U48" s="64">
+      <c r="U48" s="63">
         <f t="shared" si="7"/>
         <v>1.8603781071775227</v>
       </c>
-      <c r="V48" s="64">
+      <c r="V48" s="63">
         <f>U48</f>
         <v>1.8603781071775227</v>
       </c>

</xml_diff>